<commit_message>
Set upsilon as lambda * f (windows)
</commit_message>
<xml_diff>
--- a/src/flychams_common/config/Configuration-Heterogeneous-Benchmark.xlsx
+++ b/src/flychams_common/config/Configuration-Heterogeneous-Benchmark.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="266">
   <si>
     <t xml:space="preserve">GENERAL CONFIGURATION</t>
   </si>
@@ -628,7 +628,7 @@
     <t xml:space="preserve">Tracking Window 1.1 Multi-Window (2 Windows)</t>
   </si>
   <si>
-    <t xml:space="preserve">(480x270)</t>
+    <t xml:space="preserve">(960x540)</t>
   </si>
   <si>
     <t xml:space="preserve">MULTIWINDOW01</t>
@@ -785,9 +785,6 @@
   </si>
   <si>
     <t xml:space="preserve">Low-Resolution Tracking Camera</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(960x540)</t>
   </si>
   <si>
     <t xml:space="preserve">High-Resolution Central Camera</t>
@@ -912,9 +909,8 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="16"/>
-      <color rgb="FFFF0000"/>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -1010,7 +1006,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1063,10 +1059,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1088,6 +1080,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1730,7 +1730,7 @@
       <c r="BD3" s="12"/>
     </row>
     <row r="4" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13"/>
+      <c r="A4" s="8"/>
       <c r="B4" s="9" t="s">
         <v>21</v>
       </c>
@@ -2198,7 +2198,7 @@
       <c r="BD9" s="12"/>
     </row>
     <row r="10" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="8" t="s">
         <v>37</v>
       </c>
       <c r="B10" s="9" t="s">
@@ -2392,92 +2392,92 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="21" t="s">
         <v>216</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="22" t="s">
+        <v>256</v>
+      </c>
+      <c r="D2" s="22" t="s">
         <v>257</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="E2" s="22" t="s">
         <v>258</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="F2" s="22" t="s">
         <v>259</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="G2" s="22" t="s">
         <v>260</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="H2" s="22" t="s">
         <v>261</v>
       </c>
-      <c r="H2" s="21" t="s">
-        <v>262</v>
-      </c>
-      <c r="I2" s="21" t="s">
+      <c r="I2" s="22" t="s">
         <v>242</v>
       </c>
-      <c r="J2" s="21" t="s">
+      <c r="J2" s="22" t="s">
         <v>243</v>
       </c>
-      <c r="K2" s="21" t="s">
+      <c r="K2" s="22" t="s">
         <v>244</v>
       </c>
       <c r="L2" s="12"/>
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="B3" s="22" t="s">
-        <v>263</v>
-      </c>
-      <c r="C3" s="23" t="b">
+      <c r="B3" s="23" t="s">
+        <v>262</v>
+      </c>
+      <c r="C3" s="24" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="D3" s="22" t="s">
-        <v>264</v>
-      </c>
-      <c r="E3" s="23" t="b">
+      <c r="D3" s="23" t="s">
+        <v>263</v>
+      </c>
+      <c r="E3" s="24" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="F3" s="22" t="s">
-        <v>265</v>
-      </c>
-      <c r="G3" s="23" t="b">
+      <c r="F3" s="23" t="s">
+        <v>264</v>
+      </c>
+      <c r="G3" s="24" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H3" s="22" t="s">
-        <v>266</v>
-      </c>
-      <c r="I3" s="22" t="n">
+      <c r="H3" s="23" t="s">
+        <v>265</v>
+      </c>
+      <c r="I3" s="23" t="n">
         <v>0.4</v>
       </c>
-      <c r="J3" s="22" t="n">
+      <c r="J3" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="K3" s="22" t="n">
+      <c r="K3" s="23" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2531,12 +2531,12 @@
   </cols>
   <sheetData>
     <row r="1" s="7" customFormat="true" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
       <c r="E1" s="12"/>
       <c r="XFB1" s="3"/>
       <c r="XFC1" s="3"/>
@@ -2566,7 +2566,7 @@
       <c r="C3" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="14" t="s">
         <v>46</v>
       </c>
     </row>
@@ -2580,7 +2580,7 @@
       <c r="C4" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="14" t="s">
         <v>49</v>
       </c>
     </row>
@@ -2620,15 +2620,15 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
     </row>
     <row r="2" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
@@ -2724,7 +2724,7 @@
       <c r="D3" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="E3" s="16" t="n">
+      <c r="E3" s="15" t="n">
         <v>16</v>
       </c>
       <c r="F3" s="9" t="s">
@@ -2805,7 +2805,7 @@
       <c r="D4" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="E4" s="16" t="n">
+      <c r="E4" s="15" t="n">
         <v>16</v>
       </c>
       <c r="F4" s="9" t="s">
@@ -2885,7 +2885,7 @@
       <c r="D5" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="E5" s="16" t="n">
+      <c r="E5" s="15" t="n">
         <v>16</v>
       </c>
       <c r="F5" s="9" t="s">
@@ -3000,48 +3000,48 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="H2" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="I2" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="J2" s="18" t="s">
+      <c r="J2" s="17" t="s">
         <v>72</v>
       </c>
       <c r="L2" s="12"/>
@@ -3056,258 +3056,258 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H3" s="19" t="n">
+      <c r="H3" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I3" s="19" t="n">
+      <c r="I3" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J3" s="19" t="n">
+      <c r="J3" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="E4" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="G4" s="19" t="s">
+      <c r="G4" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H4" s="19" t="n">
+      <c r="H4" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I4" s="19" t="n">
+      <c r="I4" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J4" s="19" t="n">
+      <c r="J4" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="E5" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="F5" s="19" t="s">
+      <c r="F5" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="G5" s="19" t="s">
+      <c r="G5" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H5" s="19" t="n">
+      <c r="H5" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I5" s="19" t="n">
+      <c r="I5" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J5" s="19" t="n">
+      <c r="J5" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E6" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="F6" s="19" t="s">
+      <c r="F6" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="G6" s="19" t="s">
+      <c r="G6" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H6" s="19" t="n">
+      <c r="H6" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I6" s="19" t="n">
+      <c r="I6" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J6" s="19" t="n">
+      <c r="J6" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H7" s="19" t="n">
+      <c r="H7" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I7" s="19" t="n">
+      <c r="I7" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J7" s="19" t="n">
+      <c r="J7" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="F8" s="19" t="s">
+      <c r="F8" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="G8" s="19" t="s">
+      <c r="G8" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H8" s="19" t="n">
+      <c r="H8" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I8" s="19" t="n">
+      <c r="I8" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J8" s="19" t="n">
+      <c r="J8" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="F9" s="19" t="s">
+      <c r="F9" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="G9" s="19" t="s">
+      <c r="G9" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H9" s="19" t="n">
+      <c r="H9" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I9" s="19" t="n">
+      <c r="I9" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J9" s="19" t="n">
+      <c r="J9" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="18" t="s">
         <v>100</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="E10" s="19" t="s">
+      <c r="E10" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="F10" s="19" t="s">
+      <c r="F10" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="G10" s="19" t="s">
+      <c r="G10" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="19" t="n">
+      <c r="H10" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I10" s="19" t="n">
+      <c r="I10" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J10" s="19" t="n">
+      <c r="J10" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
@@ -3353,32 +3353,32 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="19" t="s">
         <v>105</v>
       </c>
       <c r="H2" s="12"/>
@@ -3394,22 +3394,22 @@
       <c r="XFD2" s="12"/>
     </row>
     <row r="3" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="D3" s="19" t="n">
+      <c r="D3" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E3" s="19" t="n">
+      <c r="E3" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F3" s="19" t="n">
+      <c r="F3" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G3" s="2"/>
@@ -3419,22 +3419,22 @@
       <c r="XEY3" s="3"/>
     </row>
     <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="D4" s="19" t="n">
+      <c r="D4" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E4" s="19" t="n">
+      <c r="E4" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F4" s="19" t="n">
+      <c r="F4" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G4" s="2"/>
@@ -3444,22 +3444,22 @@
       <c r="XEY4" s="3"/>
     </row>
     <row r="5" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D5" s="19" t="n">
+      <c r="D5" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E5" s="19" t="n">
+      <c r="E5" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F5" s="19" t="n">
+      <c r="F5" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G5" s="2"/>
@@ -3469,22 +3469,22 @@
       <c r="XEY5" s="3"/>
     </row>
     <row r="6" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="D6" s="19" t="n">
+      <c r="D6" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E6" s="19" t="n">
+      <c r="E6" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F6" s="19" t="n">
+      <c r="F6" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G6" s="2"/>
@@ -3494,22 +3494,22 @@
       <c r="XEY6" s="3"/>
     </row>
     <row r="7" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="D7" s="19" t="n">
+      <c r="D7" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E7" s="19" t="n">
+      <c r="E7" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F7" s="19" t="n">
+      <c r="F7" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G7" s="2"/>
@@ -3519,22 +3519,22 @@
       <c r="XEY7" s="3"/>
     </row>
     <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>116</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="D8" s="19" t="n">
+      <c r="D8" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E8" s="19" t="n">
+      <c r="E8" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F8" s="19" t="n">
+      <c r="F8" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G8" s="2"/>
@@ -3544,22 +3544,22 @@
       <c r="XEY8" s="3"/>
     </row>
     <row r="9" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="18" t="s">
         <v>118</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D9" s="19" t="n">
+      <c r="D9" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E9" s="19" t="n">
+      <c r="E9" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F9" s="19" t="n">
+      <c r="F9" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G9" s="2"/>
@@ -3569,22 +3569,22 @@
       <c r="XEY9" s="3"/>
     </row>
     <row r="10" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="D10" s="19" t="n">
+      <c r="D10" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E10" s="19" t="n">
+      <c r="E10" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F10" s="19" t="n">
+      <c r="F10" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G10" s="2"/>
@@ -3650,56 +3650,56 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
-      <c r="L1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>124</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="H2" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="I2" s="17" t="s">
         <v>125</v>
       </c>
-      <c r="J2" s="18" t="s">
+      <c r="J2" s="17" t="s">
         <v>126</v>
       </c>
-      <c r="K2" s="18" t="s">
+      <c r="K2" s="17" t="s">
         <v>127</v>
       </c>
-      <c r="L2" s="18" t="s">
+      <c r="L2" s="17" t="s">
         <v>128</v>
       </c>
       <c r="M2" s="12"/>
@@ -3712,652 +3712,652 @@
       <c r="XFC2" s="12"/>
     </row>
     <row r="3" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>129</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>130</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="H3" s="19" t="s">
+      <c r="H3" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="I3" s="19" t="n">
+      <c r="I3" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J3" s="19" t="n">
+      <c r="J3" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K3" s="19" t="n">
+      <c r="K3" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L3" s="19" t="s">
+      <c r="L3" s="18" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>137</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="18" t="s">
         <v>139</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="E4" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="G4" s="19" t="s">
+      <c r="G4" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="H4" s="19" t="s">
+      <c r="H4" s="18" t="s">
         <v>142</v>
       </c>
-      <c r="I4" s="19" t="n">
+      <c r="I4" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="J4" s="19" t="n">
+      <c r="J4" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K4" s="19" t="n">
+      <c r="K4" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L4" s="19" t="s">
+      <c r="L4" s="18" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="18" t="s">
         <v>144</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="18" t="s">
         <v>145</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="18" t="s">
         <v>139</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="E5" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="F5" s="19" t="s">
+      <c r="F5" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="G5" s="19" t="s">
+      <c r="G5" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="H5" s="19" t="s">
+      <c r="H5" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="I5" s="19" t="n">
+      <c r="I5" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="J5" s="19" t="n">
+      <c r="J5" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K5" s="19" t="n">
+      <c r="K5" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L5" s="19" t="s">
+      <c r="L5" s="18" t="s">
         <v>147</v>
       </c>
       <c r="XFD5" s="12"/>
     </row>
     <row r="6" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E6" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="F6" s="19" t="s">
+      <c r="F6" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="G6" s="19" t="s">
+      <c r="G6" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="H6" s="19" t="s">
+      <c r="H6" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="I6" s="19" t="n">
+      <c r="I6" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J6" s="19" t="n">
+      <c r="J6" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K6" s="19" t="n">
+      <c r="K6" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L6" s="19" t="s">
+      <c r="L6" s="18" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="7" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="18" t="s">
         <v>151</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="18" t="s">
         <v>139</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="H7" s="19" t="s">
+      <c r="H7" s="18" t="s">
         <v>142</v>
       </c>
-      <c r="I7" s="19" t="n">
+      <c r="I7" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="J7" s="19" t="n">
+      <c r="J7" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K7" s="19" t="n">
+      <c r="K7" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L7" s="19" t="s">
+      <c r="L7" s="18" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>155</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="18" t="s">
         <v>139</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="F8" s="19" t="s">
+      <c r="F8" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="G8" s="19" t="s">
+      <c r="G8" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="H8" s="19" t="s">
+      <c r="H8" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="I8" s="19" t="n">
+      <c r="I8" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="J8" s="19" t="n">
+      <c r="J8" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K8" s="19" t="n">
+      <c r="K8" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L8" s="19" t="s">
+      <c r="L8" s="18" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="9" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="18" t="s">
         <v>157</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="18" t="s">
         <v>158</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="F9" s="19" t="s">
+      <c r="F9" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="G9" s="19" t="s">
+      <c r="G9" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="H9" s="19" t="s">
+      <c r="H9" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="I9" s="19" t="n">
+      <c r="I9" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J9" s="19" t="n">
+      <c r="J9" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K9" s="19" t="n">
+      <c r="K9" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L9" s="19" t="s">
+      <c r="L9" s="18" t="s">
         <v>159</v>
       </c>
       <c r="XFD9" s="2"/>
     </row>
     <row r="10" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="18" t="s">
         <v>160</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="18" t="s">
         <v>139</v>
       </c>
-      <c r="E10" s="19" t="s">
+      <c r="E10" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="F10" s="19" t="s">
+      <c r="F10" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="G10" s="19" t="s">
+      <c r="G10" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="H10" s="19" t="s">
+      <c r="H10" s="18" t="s">
         <v>142</v>
       </c>
-      <c r="I10" s="19" t="n">
+      <c r="I10" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="J10" s="19" t="n">
+      <c r="J10" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K10" s="19" t="n">
+      <c r="K10" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L10" s="19" t="s">
+      <c r="L10" s="18" t="s">
         <v>162</v>
       </c>
       <c r="XFD10" s="2"/>
     </row>
     <row r="11" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="18" t="s">
         <v>163</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D11" s="19" t="s">
+      <c r="D11" s="18" t="s">
         <v>139</v>
       </c>
-      <c r="E11" s="19" t="s">
+      <c r="E11" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="F11" s="19" t="s">
+      <c r="F11" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="G11" s="19" t="s">
+      <c r="G11" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="H11" s="19" t="s">
+      <c r="H11" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="I11" s="19" t="n">
+      <c r="I11" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="J11" s="19" t="n">
+      <c r="J11" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K11" s="19" t="n">
+      <c r="K11" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L11" s="19" t="s">
+      <c r="L11" s="18" t="s">
         <v>165</v>
       </c>
       <c r="XFD11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="18" t="s">
         <v>167</v>
       </c>
-      <c r="C12" s="19" t="s">
+      <c r="C12" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="D12" s="19" t="s">
+      <c r="D12" s="18" t="s">
         <v>168</v>
       </c>
-      <c r="E12" s="19" t="s">
+      <c r="E12" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="F12" s="19" t="s">
+      <c r="F12" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="G12" s="19" t="s">
+      <c r="G12" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="H12" s="19" t="s">
+      <c r="H12" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="I12" s="19" t="n">
+      <c r="I12" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J12" s="19" t="n">
+      <c r="J12" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K12" s="19" t="n">
+      <c r="K12" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L12" s="19" t="s">
+      <c r="L12" s="18" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="18" t="s">
         <v>170</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="18" t="s">
         <v>171</v>
       </c>
-      <c r="C13" s="19" t="s">
+      <c r="C13" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="D13" s="19" t="s">
+      <c r="D13" s="18" t="s">
         <v>168</v>
       </c>
-      <c r="E13" s="19" t="s">
+      <c r="E13" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="F13" s="19" t="s">
+      <c r="F13" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="G13" s="19" t="s">
+      <c r="G13" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="H13" s="19" t="s">
+      <c r="H13" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="I13" s="19" t="n">
+      <c r="I13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J13" s="19" t="n">
+      <c r="J13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K13" s="19" t="n">
+      <c r="K13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L13" s="19" t="s">
+      <c r="L13" s="18" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="19" t="s">
+      <c r="A14" s="18" t="s">
         <v>173</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="18" t="s">
         <v>174</v>
       </c>
-      <c r="C14" s="19" t="s">
+      <c r="C14" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="D14" s="19" t="s">
+      <c r="D14" s="18" t="s">
         <v>168</v>
       </c>
-      <c r="E14" s="19" t="s">
+      <c r="E14" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="F14" s="19" t="s">
+      <c r="F14" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="G14" s="19" t="s">
+      <c r="G14" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="H14" s="19" t="s">
+      <c r="H14" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="I14" s="19" t="n">
+      <c r="I14" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J14" s="19" t="n">
+      <c r="J14" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K14" s="19" t="n">
+      <c r="K14" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L14" s="19" t="s">
+      <c r="L14" s="18" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="18" t="s">
         <v>176</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="18" t="s">
         <v>177</v>
       </c>
-      <c r="C15" s="19" t="s">
+      <c r="C15" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D15" s="19" t="s">
+      <c r="D15" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="E15" s="19" t="s">
+      <c r="E15" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="F15" s="19" t="s">
+      <c r="F15" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="G15" s="19" t="s">
+      <c r="G15" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="H15" s="19" t="s">
+      <c r="H15" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="I15" s="19" t="n">
+      <c r="I15" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J15" s="19" t="n">
+      <c r="J15" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K15" s="19" t="n">
+      <c r="K15" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L15" s="19" t="s">
+      <c r="L15" s="18" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="19" t="s">
+      <c r="A16" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="B16" s="19" t="s">
+      <c r="B16" s="18" t="s">
         <v>180</v>
       </c>
-      <c r="C16" s="19" t="s">
+      <c r="C16" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D16" s="19" t="s">
+      <c r="D16" s="18" t="s">
         <v>139</v>
       </c>
-      <c r="E16" s="19" t="s">
+      <c r="E16" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="F16" s="19" t="s">
+      <c r="F16" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="G16" s="19" t="s">
+      <c r="G16" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="H16" s="19" t="s">
+      <c r="H16" s="18" t="s">
         <v>142</v>
       </c>
-      <c r="I16" s="19" t="n">
+      <c r="I16" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="J16" s="19" t="n">
+      <c r="J16" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K16" s="19" t="n">
+      <c r="K16" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L16" s="19" t="s">
+      <c r="L16" s="18" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="19" t="s">
+      <c r="A17" s="18" t="s">
         <v>182</v>
       </c>
-      <c r="B17" s="19" t="s">
+      <c r="B17" s="18" t="s">
         <v>183</v>
       </c>
-      <c r="C17" s="19" t="s">
+      <c r="C17" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D17" s="19" t="s">
+      <c r="D17" s="18" t="s">
         <v>139</v>
       </c>
-      <c r="E17" s="19" t="s">
+      <c r="E17" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="F17" s="19" t="s">
+      <c r="F17" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="G17" s="19" t="s">
+      <c r="G17" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="H17" s="19" t="s">
+      <c r="H17" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="I17" s="19" t="n">
+      <c r="I17" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="J17" s="19" t="n">
+      <c r="J17" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K17" s="19" t="n">
+      <c r="K17" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L17" s="19" t="s">
+      <c r="L17" s="18" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="18" t="s">
         <v>185</v>
       </c>
-      <c r="B18" s="19" t="s">
+      <c r="B18" s="18" t="s">
         <v>186</v>
       </c>
-      <c r="C18" s="19" t="s">
+      <c r="C18" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D18" s="19" t="s">
+      <c r="D18" s="18" t="s">
         <v>139</v>
       </c>
-      <c r="E18" s="19" t="s">
+      <c r="E18" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="F18" s="19" t="s">
+      <c r="F18" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="G18" s="19" t="s">
+      <c r="G18" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="H18" s="19" t="s">
+      <c r="H18" s="18" t="s">
         <v>188</v>
       </c>
-      <c r="I18" s="19" t="n">
+      <c r="I18" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="J18" s="19" t="n">
+      <c r="J18" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K18" s="19" t="n">
+      <c r="K18" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L18" s="19" t="s">
+      <c r="L18" s="18" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="19" t="s">
+      <c r="A19" s="18" t="s">
         <v>190</v>
       </c>
-      <c r="B19" s="19" t="s">
+      <c r="B19" s="18" t="s">
         <v>191</v>
       </c>
-      <c r="C19" s="19" t="s">
+      <c r="C19" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="D19" s="19" t="s">
+      <c r="D19" s="18" t="s">
         <v>168</v>
       </c>
-      <c r="E19" s="19" t="s">
+      <c r="E19" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="F19" s="19" t="s">
+      <c r="F19" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="G19" s="19" t="s">
+      <c r="G19" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="H19" s="19" t="s">
+      <c r="H19" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="I19" s="19" t="n">
+      <c r="I19" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J19" s="19" t="n">
+      <c r="J19" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K19" s="19" t="n">
+      <c r="K19" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L19" s="19" t="s">
+      <c r="L19" s="18" t="s">
         <v>192</v>
       </c>
     </row>
@@ -4398,36 +4398,36 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>193</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>194</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>195</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="17" t="s">
         <v>196</v>
       </c>
       <c r="XEU2" s="3"/>
@@ -4442,209 +4442,209 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>197</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>198</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="E3" s="19" t="n">
+      <c r="E3" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F3" s="19" t="n">
+      <c r="F3" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G3" s="19" t="n">
+      <c r="G3" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>200</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>201</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="E4" s="19" t="n">
+      <c r="E4" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F4" s="19" t="n">
+      <c r="F4" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="19" t="n">
+      <c r="G4" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="18" t="s">
         <v>202</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="18" t="s">
         <v>203</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="E5" s="19" t="n">
+      <c r="E5" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F5" s="19" t="n">
+      <c r="F5" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G5" s="19" t="n">
+      <c r="G5" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>205</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="E6" s="19" t="n">
+      <c r="E6" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F6" s="19" t="n">
+      <c r="F6" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G6" s="19" t="n">
+      <c r="G6" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="18" t="s">
         <v>206</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>207</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="E7" s="19" t="n">
+      <c r="E7" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F7" s="19" t="n">
+      <c r="F7" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="19" t="n">
+      <c r="G7" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="18" t="s">
         <v>208</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>209</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="E8" s="19" t="n">
+      <c r="E8" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F8" s="19" t="n">
+      <c r="F8" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="19" t="n">
+      <c r="G8" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="18" t="s">
         <v>210</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="18" t="s">
         <v>211</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="E9" s="19" t="n">
+      <c r="E9" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F9" s="19" t="n">
+      <c r="F9" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="19" t="n">
+      <c r="G9" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="18" t="s">
         <v>212</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="18" t="s">
         <v>213</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="E10" s="19" t="n">
+      <c r="E10" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F10" s="19" t="n">
+      <c r="F10" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="19" t="n">
+      <c r="G10" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="18" t="s">
         <v>214</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="18" t="s">
         <v>215</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="D11" s="19" t="s">
+      <c r="D11" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="E11" s="19" t="n">
+      <c r="E11" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F11" s="19" t="n">
+      <c r="F11" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G11" s="19" t="n">
+      <c r="G11" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
@@ -4695,140 +4695,140 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="21" t="s">
         <v>216</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
-      <c r="O1" s="20"/>
-      <c r="P1" s="20"/>
-      <c r="Q1" s="20"/>
-      <c r="R1" s="20"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="21"/>
+      <c r="O1" s="21"/>
+      <c r="P1" s="21"/>
+      <c r="Q1" s="21"/>
+      <c r="R1" s="21"/>
     </row>
     <row r="2" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="22" t="s">
         <v>217</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="22" t="s">
         <v>218</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="22" t="s">
         <v>219</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="22" t="s">
         <v>220</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="H2" s="22" t="s">
         <v>221</v>
       </c>
-      <c r="I2" s="21" t="s">
+      <c r="I2" s="22" t="s">
         <v>222</v>
       </c>
-      <c r="J2" s="21" t="s">
+      <c r="J2" s="22" t="s">
         <v>223</v>
       </c>
-      <c r="K2" s="21" t="s">
+      <c r="K2" s="22" t="s">
         <v>224</v>
       </c>
-      <c r="L2" s="21" t="s">
+      <c r="L2" s="22" t="s">
         <v>225</v>
       </c>
-      <c r="M2" s="21" t="s">
+      <c r="M2" s="22" t="s">
         <v>226</v>
       </c>
-      <c r="N2" s="21" t="s">
+      <c r="N2" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="O2" s="21" t="s">
+      <c r="O2" s="22" t="s">
         <v>228</v>
       </c>
-      <c r="P2" s="21" t="s">
+      <c r="P2" s="22" t="s">
         <v>229</v>
       </c>
-      <c r="Q2" s="21" t="s">
+      <c r="Q2" s="22" t="s">
         <v>230</v>
       </c>
-      <c r="R2" s="21" t="s">
+      <c r="R2" s="22" t="s">
         <v>231</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="23" t="s">
         <v>76</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="23" t="s">
         <v>232</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="C3" s="23" t="s">
         <v>233</v>
       </c>
-      <c r="D3" s="22" t="n">
+      <c r="D3" s="23" t="n">
         <v>8</v>
       </c>
-      <c r="E3" s="22" t="n">
+      <c r="E3" s="23" t="n">
         <v>12</v>
       </c>
-      <c r="F3" s="23" t="b">
+      <c r="F3" s="24" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="G3" s="22" t="s">
+      <c r="G3" s="23" t="s">
         <v>234</v>
       </c>
-      <c r="H3" s="23" t="b">
+      <c r="H3" s="24" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="I3" s="22" t="s">
+      <c r="I3" s="23" t="s">
         <v>235</v>
       </c>
-      <c r="J3" s="23" t="b">
+      <c r="J3" s="24" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="K3" s="22" t="s">
+      <c r="K3" s="23" t="s">
         <v>236</v>
       </c>
-      <c r="L3" s="23" t="b">
+      <c r="L3" s="24" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="M3" s="22" t="s">
+      <c r="M3" s="23" t="s">
         <v>237</v>
       </c>
-      <c r="N3" s="22" t="n">
+      <c r="N3" s="23" t="n">
         <v>6.5</v>
       </c>
-      <c r="O3" s="22" t="n">
+      <c r="O3" s="23" t="n">
         <v>2.5</v>
       </c>
-      <c r="P3" s="22" t="n">
+      <c r="P3" s="23" t="n">
         <v>400</v>
       </c>
-      <c r="Q3" s="22" t="n">
+      <c r="Q3" s="23" t="n">
         <v>350</v>
       </c>
-      <c r="R3" s="22" t="n">
+      <c r="R3" s="23" t="n">
         <v>25</v>
       </c>
     </row>
@@ -4888,52 +4888,52 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="21" t="s">
         <v>216</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="22" t="s">
         <v>193</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="22" t="s">
         <v>238</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="22" t="s">
         <v>239</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="22" t="s">
         <v>240</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="H2" s="22" t="s">
         <v>241</v>
       </c>
-      <c r="I2" s="21" t="s">
+      <c r="I2" s="22" t="s">
         <v>242</v>
       </c>
-      <c r="J2" s="21" t="s">
+      <c r="J2" s="22" t="s">
         <v>243</v>
       </c>
-      <c r="K2" s="21" t="s">
+      <c r="K2" s="22" t="s">
         <v>244</v>
       </c>
       <c r="XFB2" s="3"/>
@@ -4941,110 +4941,110 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="23" t="s">
         <v>131</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="23" t="s">
         <v>245</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="C3" s="23" t="s">
         <v>246</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="23" t="s">
         <v>247</v>
       </c>
-      <c r="E3" s="22" t="s">
+      <c r="E3" s="23" t="s">
         <v>248</v>
       </c>
-      <c r="F3" s="22" t="s">
+      <c r="F3" s="23" t="s">
         <v>249</v>
       </c>
-      <c r="G3" s="23" t="b">
+      <c r="G3" s="24" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H3" s="22" t="s">
+      <c r="H3" s="23" t="s">
         <v>250</v>
       </c>
-      <c r="I3" s="22" t="n">
+      <c r="I3" s="23" t="n">
         <v>0.5</v>
       </c>
-      <c r="J3" s="22" t="n">
+      <c r="J3" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="K3" s="22" t="n">
+      <c r="K3" s="23" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="23" t="s">
         <v>139</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="23" t="s">
         <v>251</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="23" t="s">
         <v>246</v>
       </c>
-      <c r="D4" s="22" t="s">
-        <v>252</v>
-      </c>
-      <c r="E4" s="22" t="s">
+      <c r="D4" s="23" t="s">
+        <v>199</v>
+      </c>
+      <c r="E4" s="23" t="s">
         <v>248</v>
       </c>
-      <c r="F4" s="22" t="s">
+      <c r="F4" s="23" t="s">
         <v>249</v>
       </c>
-      <c r="G4" s="23" t="b">
+      <c r="G4" s="24" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H4" s="22" t="s">
+      <c r="H4" s="23" t="s">
         <v>250</v>
       </c>
-      <c r="I4" s="22" t="n">
+      <c r="I4" s="23" t="n">
         <v>0.5</v>
       </c>
-      <c r="J4" s="22" t="n">
+      <c r="J4" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="K4" s="22" t="n">
+      <c r="K4" s="23" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="23" t="s">
         <v>168</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="23" t="s">
+        <v>252</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>246</v>
+      </c>
+      <c r="D5" s="23" t="s">
         <v>253</v>
       </c>
-      <c r="C5" s="22" t="s">
-        <v>246</v>
-      </c>
-      <c r="D5" s="22" t="s">
+      <c r="E5" s="23" t="s">
+        <v>248</v>
+      </c>
+      <c r="F5" s="23" t="s">
         <v>254</v>
       </c>
-      <c r="E5" s="22" t="s">
-        <v>248</v>
-      </c>
-      <c r="F5" s="22" t="s">
-        <v>255</v>
-      </c>
-      <c r="G5" s="23" t="b">
+      <c r="G5" s="24" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H5" s="22" t="s">
-        <v>256</v>
-      </c>
-      <c r="I5" s="22" t="n">
+      <c r="H5" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="I5" s="23" t="n">
         <v>0.5</v>
       </c>
-      <c r="J5" s="22" t="n">
+      <c r="J5" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="K5" s="22" t="n">
+      <c r="K5" s="23" t="n">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve agent positioning costs
</commit_message>
<xml_diff>
--- a/src/flychams_common/config/Configuration-Heterogeneous-Benchmark.xlsx
+++ b/src/flychams_common/config/Configuration-Heterogeneous-Benchmark.xlsx
@@ -64,6 +64,9 @@
     <t xml:space="preserve">StartHour</t>
   </si>
   <si>
+    <t xml:space="preserve">X</t>
+  </si>
+  <si>
     <t xml:space="preserve">MISSION00</t>
   </si>
   <si>
@@ -82,7 +85,7 @@
     <t xml:space="preserve">(-200.0, 200.0)</t>
   </si>
   <si>
-    <t xml:space="preserve">(15.0, 150.0)</t>
+    <t xml:space="preserve">(30.0, 150.0)</t>
   </si>
   <si>
     <t xml:space="preserve">PX4</t>
@@ -140,9 +143,6 @@
   </si>
   <si>
     <t xml:space="preserve">GROUP02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">X</t>
   </si>
   <si>
     <t xml:space="preserve">MISSION07</t>
@@ -902,17 +902,18 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="16"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color theme="2" tint="-0.75"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">
@@ -1006,7 +1007,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1039,7 +1040,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1051,12 +1052,16 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -1080,14 +1085,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1652,36 +1649,38 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8"/>
+      <c r="A3" s="8" t="s">
+        <v>11</v>
+      </c>
       <c r="B3" s="9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I3" s="11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L3" s="12"/>
       <c r="M3" s="12"/>
@@ -1730,36 +1729,36 @@
       <c r="BD3" s="12"/>
     </row>
     <row r="4" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8"/>
+      <c r="A4" s="13"/>
       <c r="B4" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="J4" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="K4" s="9" t="s">
         <v>21</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="G4" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="H4" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="I4" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="J4" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="K4" s="9" t="s">
-        <v>20</v>
       </c>
       <c r="L4" s="12"/>
       <c r="M4" s="12"/>
@@ -1808,36 +1807,36 @@
       <c r="BD4" s="12"/>
     </row>
     <row r="5" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8"/>
+      <c r="A5" s="13"/>
       <c r="B5" s="9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J5" s="9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L5" s="12"/>
       <c r="M5" s="12"/>
@@ -1886,36 +1885,36 @@
       <c r="BD5" s="12"/>
     </row>
     <row r="6" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8"/>
+      <c r="A6" s="13"/>
       <c r="B6" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L6" s="12"/>
       <c r="M6" s="12"/>
@@ -1964,36 +1963,36 @@
       <c r="BD6" s="12"/>
     </row>
     <row r="7" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8"/>
+      <c r="A7" s="13"/>
       <c r="B7" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>29</v>
-      </c>
       <c r="F7" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J7" s="9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K7" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L7" s="12"/>
       <c r="M7" s="12"/>
@@ -2042,36 +2041,36 @@
       <c r="BD7" s="12"/>
     </row>
     <row r="8" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8"/>
+      <c r="A8" s="13"/>
       <c r="B8" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J8" s="9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L8" s="12"/>
       <c r="M8" s="12"/>
@@ -2120,36 +2119,36 @@
       <c r="BD8" s="12"/>
     </row>
     <row r="9" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8"/>
+      <c r="A9" s="13"/>
       <c r="B9" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I9" s="11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J9" s="9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K9" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L9" s="12"/>
       <c r="M9" s="12"/>
@@ -2198,9 +2197,7 @@
       <c r="BD9" s="12"/>
     </row>
     <row r="10" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="s">
-        <v>37</v>
-      </c>
+      <c r="A10" s="13"/>
       <c r="B10" s="9" t="s">
         <v>38</v>
       </c>
@@ -2208,28 +2205,28 @@
         <v>39</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J10" s="9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K10" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L10" s="12"/>
       <c r="M10" s="12"/>
@@ -2278,7 +2275,7 @@
       <c r="BD10" s="12"/>
     </row>
     <row r="11" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8"/>
+      <c r="A11" s="13"/>
       <c r="B11" s="9" t="s">
         <v>40</v>
       </c>
@@ -2286,28 +2283,28 @@
         <v>41</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H11" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I11" s="11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J11" s="9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K11" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L11" s="12"/>
       <c r="M11" s="12"/>
@@ -2392,92 +2389,92 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="20" t="s">
         <v>216</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="22" t="s">
+      <c r="C2" s="21" t="s">
         <v>256</v>
       </c>
-      <c r="D2" s="22" t="s">
+      <c r="D2" s="21" t="s">
         <v>257</v>
       </c>
-      <c r="E2" s="22" t="s">
+      <c r="E2" s="21" t="s">
         <v>258</v>
       </c>
-      <c r="F2" s="22" t="s">
+      <c r="F2" s="21" t="s">
         <v>259</v>
       </c>
-      <c r="G2" s="22" t="s">
+      <c r="G2" s="21" t="s">
         <v>260</v>
       </c>
-      <c r="H2" s="22" t="s">
+      <c r="H2" s="21" t="s">
         <v>261</v>
       </c>
-      <c r="I2" s="22" t="s">
+      <c r="I2" s="21" t="s">
         <v>242</v>
       </c>
-      <c r="J2" s="22" t="s">
+      <c r="J2" s="21" t="s">
         <v>243</v>
       </c>
-      <c r="K2" s="22" t="s">
+      <c r="K2" s="21" t="s">
         <v>244</v>
       </c>
       <c r="L2" s="12"/>
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="22" t="s">
         <v>132</v>
       </c>
-      <c r="B3" s="23" t="s">
+      <c r="B3" s="22" t="s">
         <v>262</v>
       </c>
-      <c r="C3" s="24" t="b">
+      <c r="C3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="D3" s="23" t="s">
+      <c r="D3" s="22" t="s">
         <v>263</v>
       </c>
-      <c r="E3" s="24" t="b">
+      <c r="E3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="F3" s="23" t="s">
+      <c r="F3" s="22" t="s">
         <v>264</v>
       </c>
-      <c r="G3" s="24" t="b">
+      <c r="G3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H3" s="23" t="s">
+      <c r="H3" s="22" t="s">
         <v>265</v>
       </c>
-      <c r="I3" s="23" t="n">
+      <c r="I3" s="22" t="n">
         <v>0.4</v>
       </c>
-      <c r="J3" s="23" t="n">
+      <c r="J3" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="K3" s="23" t="n">
+      <c r="K3" s="22" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2531,12 +2528,12 @@
   </cols>
   <sheetData>
     <row r="1" s="7" customFormat="true" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
       <c r="E1" s="12"/>
       <c r="XFB1" s="3"/>
       <c r="XFC1" s="3"/>
@@ -2558,7 +2555,7 @@
     </row>
     <row r="3" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>44</v>
@@ -2566,7 +2563,7 @@
       <c r="C3" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="15" t="s">
         <v>46</v>
       </c>
     </row>
@@ -2580,7 +2577,7 @@
       <c r="C4" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="15" t="s">
         <v>49</v>
       </c>
     </row>
@@ -2620,15 +2617,15 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
     </row>
     <row r="2" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
@@ -2719,12 +2716,12 @@
         <v>55</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="E3" s="15" t="n">
+      <c r="E3" s="16" t="n">
         <v>16</v>
       </c>
       <c r="F3" s="9" t="s">
@@ -2800,12 +2797,12 @@
         <v>60</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D4" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="E4" s="15" t="n">
+      <c r="E4" s="16" t="n">
         <v>16</v>
       </c>
       <c r="F4" s="9" t="s">
@@ -2880,12 +2877,12 @@
         <v>63</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="E5" s="15" t="n">
+      <c r="E5" s="16" t="n">
         <v>16</v>
       </c>
       <c r="F5" s="9" t="s">
@@ -3000,48 +2997,48 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="F2" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="G2" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="H2" s="17" t="s">
+      <c r="H2" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="I2" s="17" t="s">
+      <c r="I2" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="J2" s="17" t="s">
+      <c r="J2" s="18" t="s">
         <v>72</v>
       </c>
       <c r="L2" s="12"/>
@@ -3056,258 +3053,258 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="C3" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" s="18" t="s">
+      <c r="C3" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="G3" s="18" t="s">
+      <c r="G3" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="H3" s="18" t="n">
+      <c r="H3" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I3" s="18" t="n">
+      <c r="I3" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J3" s="18" t="n">
+      <c r="J3" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="19" t="s">
         <v>79</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="19" t="s">
         <v>80</v>
       </c>
-      <c r="C4" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" s="18" t="s">
+      <c r="C4" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="E4" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="F4" s="18" t="s">
+      <c r="F4" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="G4" s="18" t="s">
+      <c r="G4" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="H4" s="18" t="n">
+      <c r="H4" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I4" s="18" t="n">
+      <c r="I4" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J4" s="18" t="n">
+      <c r="J4" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="19" t="s">
         <v>84</v>
       </c>
-      <c r="C5" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="18" t="s">
+      <c r="C5" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="E5" s="18" t="s">
+      <c r="E5" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="F5" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="G5" s="18" t="s">
+      <c r="G5" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="H5" s="18" t="n">
+      <c r="H5" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I5" s="18" t="n">
+      <c r="I5" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J5" s="18" t="n">
+      <c r="J5" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="C6" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="18" t="s">
+      <c r="C6" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="E6" s="18" t="s">
+      <c r="E6" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="F6" s="18" t="s">
+      <c r="F6" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="G6" s="18" t="s">
+      <c r="G6" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="H6" s="18" t="n">
+      <c r="H6" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I6" s="18" t="n">
+      <c r="I6" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J6" s="18" t="n">
+      <c r="J6" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="C7" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="D7" s="18" t="s">
+      <c r="C7" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="E7" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="F7" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="G7" s="18" t="s">
+      <c r="G7" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="H7" s="18" t="n">
+      <c r="H7" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I7" s="18" t="n">
+      <c r="I7" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J7" s="18" t="n">
+      <c r="J7" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="19" t="s">
         <v>93</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="C8" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" s="18" t="s">
+      <c r="C8" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" s="19" t="s">
         <v>95</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="E8" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="F8" s="18" t="s">
+      <c r="F8" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="G8" s="18" t="s">
+      <c r="G8" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="H8" s="18" t="n">
+      <c r="H8" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I8" s="18" t="n">
+      <c r="I8" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J8" s="18" t="n">
+      <c r="J8" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="C9" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="D9" s="18" t="s">
+      <c r="C9" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="19" t="s">
         <v>98</v>
       </c>
-      <c r="E9" s="18" t="s">
+      <c r="E9" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="F9" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="G9" s="18" t="s">
+      <c r="G9" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="H9" s="18" t="n">
+      <c r="H9" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I9" s="18" t="n">
+      <c r="I9" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J9" s="18" t="n">
+      <c r="J9" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="C10" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="D10" s="18" t="s">
+      <c r="C10" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="E10" s="18" t="s">
+      <c r="E10" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="F10" s="18" t="s">
+      <c r="F10" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="G10" s="18" t="s">
+      <c r="G10" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="18" t="n">
+      <c r="H10" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I10" s="18" t="n">
+      <c r="I10" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J10" s="18" t="n">
+      <c r="J10" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
@@ -3353,32 +3350,32 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="D2" s="19" t="s">
+      <c r="D2" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="E2" s="19" t="s">
+      <c r="E2" s="18" t="s">
         <v>104</v>
       </c>
-      <c r="F2" s="19" t="s">
+      <c r="F2" s="18" t="s">
         <v>105</v>
       </c>
       <c r="H2" s="12"/>
@@ -3394,22 +3391,22 @@
       <c r="XFD2" s="12"/>
     </row>
     <row r="3" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="D3" s="18" t="n">
+      <c r="D3" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E3" s="18" t="n">
+      <c r="E3" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F3" s="18" t="n">
+      <c r="F3" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G3" s="2"/>
@@ -3419,22 +3416,22 @@
       <c r="XEY3" s="3"/>
     </row>
     <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="D4" s="18" t="n">
+      <c r="D4" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E4" s="18" t="n">
+      <c r="E4" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F4" s="18" t="n">
+      <c r="F4" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G4" s="2"/>
@@ -3444,22 +3441,22 @@
       <c r="XEY4" s="3"/>
     </row>
     <row r="5" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="19" t="s">
         <v>110</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="D5" s="18" t="n">
+      <c r="D5" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E5" s="18" t="n">
+      <c r="E5" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F5" s="18" t="n">
+      <c r="F5" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G5" s="2"/>
@@ -3469,22 +3466,22 @@
       <c r="XEY5" s="3"/>
     </row>
     <row r="6" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="D6" s="18" t="n">
+      <c r="D6" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E6" s="18" t="n">
+      <c r="E6" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F6" s="18" t="n">
+      <c r="F6" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G6" s="2"/>
@@ -3494,22 +3491,22 @@
       <c r="XEY6" s="3"/>
     </row>
     <row r="7" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="D7" s="18" t="n">
+      <c r="D7" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E7" s="18" t="n">
+      <c r="E7" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F7" s="18" t="n">
+      <c r="F7" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G7" s="2"/>
@@ -3519,22 +3516,22 @@
       <c r="XEY7" s="3"/>
     </row>
     <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="19" t="s">
         <v>95</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="19" t="s">
         <v>116</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="D8" s="18" t="n">
+      <c r="D8" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E8" s="18" t="n">
+      <c r="E8" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F8" s="18" t="n">
+      <c r="F8" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G8" s="2"/>
@@ -3544,22 +3541,22 @@
       <c r="XEY8" s="3"/>
     </row>
     <row r="9" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="19" t="s">
         <v>98</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="D9" s="18" t="n">
+      <c r="D9" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E9" s="18" t="n">
+      <c r="E9" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F9" s="18" t="n">
+      <c r="F9" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G9" s="2"/>
@@ -3569,22 +3566,22 @@
       <c r="XEY9" s="3"/>
     </row>
     <row r="10" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="D10" s="18" t="n">
+      <c r="D10" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E10" s="18" t="n">
+      <c r="E10" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F10" s="18" t="n">
+      <c r="F10" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G10" s="2"/>
@@ -3650,56 +3647,56 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-      <c r="L1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="F2" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="G2" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="H2" s="17" t="s">
+      <c r="H2" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="I2" s="17" t="s">
+      <c r="I2" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="J2" s="17" t="s">
+      <c r="J2" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="K2" s="17" t="s">
+      <c r="K2" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="L2" s="17" t="s">
+      <c r="L2" s="18" t="s">
         <v>128</v>
       </c>
       <c r="M2" s="12"/>
@@ -3712,652 +3709,652 @@
       <c r="XFC2" s="12"/>
     </row>
     <row r="3" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="19" t="s">
         <v>129</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="19" t="s">
         <v>130</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="G3" s="18" t="s">
+      <c r="G3" s="19" t="s">
         <v>134</v>
       </c>
-      <c r="H3" s="18" t="s">
+      <c r="H3" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="I3" s="18" t="n">
+      <c r="I3" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J3" s="18" t="n">
+      <c r="J3" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K3" s="18" t="n">
+      <c r="K3" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L3" s="18" t="s">
+      <c r="L3" s="19" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="19" t="s">
         <v>137</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="19" t="s">
         <v>138</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="D4" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="E4" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F4" s="18" t="s">
+      <c r="F4" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="G4" s="18" t="s">
+      <c r="G4" s="19" t="s">
         <v>141</v>
       </c>
-      <c r="H4" s="18" t="s">
+      <c r="H4" s="19" t="s">
         <v>142</v>
       </c>
-      <c r="I4" s="18" t="n">
+      <c r="I4" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J4" s="18" t="n">
+      <c r="J4" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K4" s="18" t="n">
+      <c r="K4" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L4" s="18" t="s">
+      <c r="L4" s="19" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="19" t="s">
         <v>144</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="19" t="s">
         <v>145</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="E5" s="18" t="s">
+      <c r="E5" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="F5" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="G5" s="18" t="s">
+      <c r="G5" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="H5" s="18" t="s">
+      <c r="H5" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="I5" s="18" t="n">
+      <c r="I5" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J5" s="18" t="n">
+      <c r="J5" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K5" s="18" t="n">
+      <c r="K5" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L5" s="18" t="s">
+      <c r="L5" s="19" t="s">
         <v>147</v>
       </c>
       <c r="XFD5" s="12"/>
     </row>
     <row r="6" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="19" t="s">
         <v>148</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="19" t="s">
         <v>149</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="E6" s="18" t="s">
+      <c r="E6" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F6" s="18" t="s">
+      <c r="F6" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="G6" s="18" t="s">
+      <c r="G6" s="19" t="s">
         <v>134</v>
       </c>
-      <c r="H6" s="18" t="s">
+      <c r="H6" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="I6" s="18" t="n">
+      <c r="I6" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J6" s="18" t="n">
+      <c r="J6" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K6" s="18" t="n">
+      <c r="K6" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L6" s="18" t="s">
+      <c r="L6" s="19" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="7" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="19" t="s">
         <v>151</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="19" t="s">
         <v>152</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="E7" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="F7" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="G7" s="18" t="s">
+      <c r="G7" s="19" t="s">
         <v>141</v>
       </c>
-      <c r="H7" s="18" t="s">
+      <c r="H7" s="19" t="s">
         <v>142</v>
       </c>
-      <c r="I7" s="18" t="n">
+      <c r="I7" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J7" s="18" t="n">
+      <c r="J7" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K7" s="18" t="n">
+      <c r="K7" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L7" s="18" t="s">
+      <c r="L7" s="19" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="19" t="s">
         <v>154</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="19" t="s">
         <v>155</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="D8" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="E8" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F8" s="18" t="s">
+      <c r="F8" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="G8" s="18" t="s">
+      <c r="G8" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="H8" s="18" t="s">
+      <c r="H8" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="I8" s="18" t="n">
+      <c r="I8" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J8" s="18" t="n">
+      <c r="J8" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K8" s="18" t="n">
+      <c r="K8" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L8" s="18" t="s">
+      <c r="L8" s="19" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="9" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="19" t="s">
         <v>157</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="19" t="s">
         <v>158</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="E9" s="18" t="s">
+      <c r="E9" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="F9" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="G9" s="18" t="s">
+      <c r="G9" s="19" t="s">
         <v>134</v>
       </c>
-      <c r="H9" s="18" t="s">
+      <c r="H9" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="I9" s="18" t="n">
+      <c r="I9" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J9" s="18" t="n">
+      <c r="J9" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K9" s="18" t="n">
+      <c r="K9" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L9" s="18" t="s">
+      <c r="L9" s="19" t="s">
         <v>159</v>
       </c>
       <c r="XFD9" s="2"/>
     </row>
     <row r="10" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="19" t="s">
         <v>160</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="19" t="s">
         <v>161</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="D10" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="E10" s="18" t="s">
+      <c r="E10" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F10" s="18" t="s">
+      <c r="F10" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="G10" s="18" t="s">
+      <c r="G10" s="19" t="s">
         <v>141</v>
       </c>
-      <c r="H10" s="18" t="s">
+      <c r="H10" s="19" t="s">
         <v>142</v>
       </c>
-      <c r="I10" s="18" t="n">
+      <c r="I10" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J10" s="18" t="n">
+      <c r="J10" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K10" s="18" t="n">
+      <c r="K10" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L10" s="18" t="s">
+      <c r="L10" s="19" t="s">
         <v>162</v>
       </c>
       <c r="XFD10" s="2"/>
     </row>
     <row r="11" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="19" t="s">
         <v>163</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="19" t="s">
         <v>164</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="D11" s="18" t="s">
+      <c r="D11" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="E11" s="18" t="s">
+      <c r="E11" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="F11" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="G11" s="18" t="s">
+      <c r="G11" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="H11" s="18" t="s">
+      <c r="H11" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="I11" s="18" t="n">
+      <c r="I11" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J11" s="18" t="n">
+      <c r="J11" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K11" s="18" t="n">
+      <c r="K11" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L11" s="18" t="s">
+      <c r="L11" s="19" t="s">
         <v>165</v>
       </c>
       <c r="XFD11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="19" t="s">
         <v>166</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="D12" s="18" t="s">
+      <c r="D12" s="19" t="s">
         <v>168</v>
       </c>
-      <c r="E12" s="18" t="s">
+      <c r="E12" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F12" s="18" t="s">
+      <c r="F12" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="G12" s="18" t="s">
+      <c r="G12" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="H12" s="18" t="s">
+      <c r="H12" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="I12" s="18" t="n">
+      <c r="I12" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J12" s="18" t="n">
+      <c r="J12" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K12" s="18" t="n">
+      <c r="K12" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L12" s="18" t="s">
+      <c r="L12" s="19" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="18" t="s">
+      <c r="A13" s="19" t="s">
         <v>170</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="19" t="s">
         <v>171</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="D13" s="18" t="s">
+      <c r="D13" s="19" t="s">
         <v>168</v>
       </c>
-      <c r="E13" s="18" t="s">
+      <c r="E13" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F13" s="18" t="s">
+      <c r="F13" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="G13" s="18" t="s">
+      <c r="G13" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="H13" s="18" t="s">
+      <c r="H13" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="I13" s="18" t="n">
+      <c r="I13" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J13" s="18" t="n">
+      <c r="J13" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K13" s="18" t="n">
+      <c r="K13" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L13" s="18" t="s">
+      <c r="L13" s="19" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="18" t="s">
+      <c r="A14" s="19" t="s">
         <v>173</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="19" t="s">
         <v>174</v>
       </c>
-      <c r="C14" s="18" t="s">
+      <c r="C14" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="D14" s="18" t="s">
+      <c r="D14" s="19" t="s">
         <v>168</v>
       </c>
-      <c r="E14" s="18" t="s">
+      <c r="E14" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F14" s="18" t="s">
+      <c r="F14" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="G14" s="18" t="s">
+      <c r="G14" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="H14" s="18" t="s">
+      <c r="H14" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="I14" s="18" t="n">
+      <c r="I14" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J14" s="18" t="n">
+      <c r="J14" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K14" s="18" t="n">
+      <c r="K14" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L14" s="18" t="s">
+      <c r="L14" s="19" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="18" t="s">
+      <c r="A15" s="19" t="s">
         <v>176</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="19" t="s">
         <v>177</v>
       </c>
-      <c r="C15" s="18" t="s">
+      <c r="C15" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="D15" s="18" t="s">
+      <c r="D15" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="E15" s="18" t="s">
+      <c r="E15" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F15" s="18" t="s">
+      <c r="F15" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="G15" s="18" t="s">
+      <c r="G15" s="19" t="s">
         <v>134</v>
       </c>
-      <c r="H15" s="18" t="s">
+      <c r="H15" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="I15" s="18" t="n">
+      <c r="I15" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J15" s="18" t="n">
+      <c r="J15" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K15" s="18" t="n">
+      <c r="K15" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L15" s="18" t="s">
+      <c r="L15" s="19" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="18" t="s">
+      <c r="A16" s="19" t="s">
         <v>179</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="B16" s="19" t="s">
         <v>180</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="C16" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="D16" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="E16" s="18" t="s">
+      <c r="E16" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F16" s="18" t="s">
+      <c r="F16" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="G16" s="18" t="s">
+      <c r="G16" s="19" t="s">
         <v>141</v>
       </c>
-      <c r="H16" s="18" t="s">
+      <c r="H16" s="19" t="s">
         <v>142</v>
       </c>
-      <c r="I16" s="18" t="n">
+      <c r="I16" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J16" s="18" t="n">
+      <c r="J16" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K16" s="18" t="n">
+      <c r="K16" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L16" s="18" t="s">
+      <c r="L16" s="19" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="18" t="s">
+      <c r="A17" s="19" t="s">
         <v>182</v>
       </c>
-      <c r="B17" s="18" t="s">
+      <c r="B17" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="D17" s="18" t="s">
+      <c r="D17" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="E17" s="18" t="s">
+      <c r="E17" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F17" s="18" t="s">
+      <c r="F17" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="G17" s="18" t="s">
+      <c r="G17" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="H17" s="18" t="s">
+      <c r="H17" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="I17" s="18" t="n">
+      <c r="I17" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J17" s="18" t="n">
+      <c r="J17" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K17" s="18" t="n">
+      <c r="K17" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L17" s="18" t="s">
+      <c r="L17" s="19" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="18" t="s">
+      <c r="A18" s="19" t="s">
         <v>185</v>
       </c>
-      <c r="B18" s="18" t="s">
+      <c r="B18" s="19" t="s">
         <v>186</v>
       </c>
-      <c r="C18" s="18" t="s">
+      <c r="C18" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="D18" s="18" t="s">
+      <c r="D18" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="E18" s="18" t="s">
+      <c r="E18" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F18" s="18" t="s">
+      <c r="F18" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="G18" s="18" t="s">
+      <c r="G18" s="19" t="s">
         <v>187</v>
       </c>
-      <c r="H18" s="18" t="s">
+      <c r="H18" s="19" t="s">
         <v>188</v>
       </c>
-      <c r="I18" s="18" t="n">
+      <c r="I18" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J18" s="18" t="n">
+      <c r="J18" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K18" s="18" t="n">
+      <c r="K18" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L18" s="18" t="s">
+      <c r="L18" s="19" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="18" t="s">
+      <c r="A19" s="19" t="s">
         <v>190</v>
       </c>
-      <c r="B19" s="18" t="s">
+      <c r="B19" s="19" t="s">
         <v>191</v>
       </c>
-      <c r="C19" s="18" t="s">
+      <c r="C19" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="D19" s="18" t="s">
+      <c r="D19" s="19" t="s">
         <v>168</v>
       </c>
-      <c r="E19" s="18" t="s">
+      <c r="E19" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F19" s="18" t="s">
+      <c r="F19" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="G19" s="18" t="s">
+      <c r="G19" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="H19" s="18" t="s">
+      <c r="H19" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="I19" s="18" t="n">
+      <c r="I19" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J19" s="18" t="n">
+      <c r="J19" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K19" s="18" t="n">
+      <c r="K19" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L19" s="18" t="s">
+      <c r="L19" s="19" t="s">
         <v>192</v>
       </c>
     </row>
@@ -4398,36 +4395,36 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="18" t="s">
         <v>193</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" s="18" t="s">
         <v>194</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="F2" s="18" t="s">
         <v>195</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="G2" s="18" t="s">
         <v>196</v>
       </c>
       <c r="XEU2" s="3"/>
@@ -4442,209 +4439,209 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="19" t="s">
         <v>197</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="D3" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="E3" s="18" t="n">
+      <c r="E3" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F3" s="18" t="n">
+      <c r="F3" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G3" s="18" t="n">
+      <c r="G3" s="19" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="19" t="s">
         <v>200</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="19" t="s">
         <v>201</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="D4" s="20" t="s">
+      <c r="D4" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="E4" s="18" t="n">
+      <c r="E4" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F4" s="18" t="n">
+      <c r="F4" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="18" t="n">
+      <c r="G4" s="19" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="19" t="s">
         <v>202</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="19" t="s">
         <v>203</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="E5" s="18" t="n">
+      <c r="E5" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F5" s="18" t="n">
+      <c r="F5" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G5" s="18" t="n">
+      <c r="G5" s="19" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="19" t="s">
         <v>204</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="19" t="s">
         <v>205</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="E6" s="18" t="n">
+      <c r="E6" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F6" s="18" t="n">
+      <c r="F6" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G6" s="18" t="n">
+      <c r="G6" s="19" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="19" t="s">
         <v>206</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="19" t="s">
         <v>207</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="D7" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="E7" s="18" t="n">
+      <c r="E7" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F7" s="18" t="n">
+      <c r="F7" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="18" t="n">
+      <c r="G7" s="19" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="19" t="s">
         <v>208</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="19" t="s">
         <v>209</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="D8" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="E8" s="18" t="n">
+      <c r="E8" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F8" s="18" t="n">
+      <c r="F8" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="18" t="n">
+      <c r="G8" s="19" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="19" t="s">
         <v>210</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="19" t="s">
         <v>211</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="D9" s="20" t="s">
+      <c r="D9" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="E9" s="18" t="n">
+      <c r="E9" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F9" s="18" t="n">
+      <c r="F9" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="18" t="n">
+      <c r="G9" s="19" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="19" t="s">
         <v>212</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="19" t="s">
         <v>213</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="D10" s="20" t="s">
+      <c r="D10" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="E10" s="18" t="n">
+      <c r="E10" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F10" s="18" t="n">
+      <c r="F10" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="18" t="n">
+      <c r="G10" s="19" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="19" t="s">
         <v>214</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="19" t="s">
         <v>215</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="D11" s="20" t="s">
+      <c r="D11" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="E11" s="18" t="n">
+      <c r="E11" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F11" s="18" t="n">
+      <c r="F11" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G11" s="18" t="n">
+      <c r="G11" s="19" t="n">
         <v>0.583</v>
       </c>
     </row>
@@ -4695,140 +4692,140 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="20" t="s">
         <v>216</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-      <c r="L1" s="21"/>
-      <c r="M1" s="21"/>
-      <c r="N1" s="21"/>
-      <c r="O1" s="21"/>
-      <c r="P1" s="21"/>
-      <c r="Q1" s="21"/>
-      <c r="R1" s="21"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="20"/>
+      <c r="N1" s="20"/>
+      <c r="O1" s="20"/>
+      <c r="P1" s="20"/>
+      <c r="Q1" s="20"/>
+      <c r="R1" s="20"/>
     </row>
     <row r="2" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="22" t="s">
+      <c r="C2" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="D2" s="22" t="s">
+      <c r="D2" s="21" t="s">
         <v>217</v>
       </c>
-      <c r="E2" s="22" t="s">
+      <c r="E2" s="21" t="s">
         <v>218</v>
       </c>
-      <c r="F2" s="22" t="s">
+      <c r="F2" s="21" t="s">
         <v>219</v>
       </c>
-      <c r="G2" s="22" t="s">
+      <c r="G2" s="21" t="s">
         <v>220</v>
       </c>
-      <c r="H2" s="22" t="s">
+      <c r="H2" s="21" t="s">
         <v>221</v>
       </c>
-      <c r="I2" s="22" t="s">
+      <c r="I2" s="21" t="s">
         <v>222</v>
       </c>
-      <c r="J2" s="22" t="s">
+      <c r="J2" s="21" t="s">
         <v>223</v>
       </c>
-      <c r="K2" s="22" t="s">
+      <c r="K2" s="21" t="s">
         <v>224</v>
       </c>
-      <c r="L2" s="22" t="s">
+      <c r="L2" s="21" t="s">
         <v>225</v>
       </c>
-      <c r="M2" s="22" t="s">
+      <c r="M2" s="21" t="s">
         <v>226</v>
       </c>
-      <c r="N2" s="22" t="s">
+      <c r="N2" s="21" t="s">
         <v>227</v>
       </c>
-      <c r="O2" s="22" t="s">
+      <c r="O2" s="21" t="s">
         <v>228</v>
       </c>
-      <c r="P2" s="22" t="s">
+      <c r="P2" s="21" t="s">
         <v>229</v>
       </c>
-      <c r="Q2" s="22" t="s">
+      <c r="Q2" s="21" t="s">
         <v>230</v>
       </c>
-      <c r="R2" s="22" t="s">
+      <c r="R2" s="21" t="s">
         <v>231</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="B3" s="23" t="s">
+      <c r="B3" s="22" t="s">
         <v>232</v>
       </c>
-      <c r="C3" s="23" t="s">
+      <c r="C3" s="22" t="s">
         <v>233</v>
       </c>
-      <c r="D3" s="23" t="n">
+      <c r="D3" s="22" t="n">
         <v>8</v>
       </c>
-      <c r="E3" s="23" t="n">
+      <c r="E3" s="22" t="n">
         <v>12</v>
       </c>
-      <c r="F3" s="24" t="b">
+      <c r="F3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="G3" s="23" t="s">
+      <c r="G3" s="22" t="s">
         <v>234</v>
       </c>
-      <c r="H3" s="24" t="b">
+      <c r="H3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="I3" s="23" t="s">
+      <c r="I3" s="22" t="s">
         <v>235</v>
       </c>
-      <c r="J3" s="24" t="b">
+      <c r="J3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="K3" s="23" t="s">
+      <c r="K3" s="22" t="s">
         <v>236</v>
       </c>
-      <c r="L3" s="24" t="b">
+      <c r="L3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="M3" s="23" t="s">
+      <c r="M3" s="22" t="s">
         <v>237</v>
       </c>
-      <c r="N3" s="23" t="n">
+      <c r="N3" s="22" t="n">
         <v>6.5</v>
       </c>
-      <c r="O3" s="23" t="n">
+      <c r="O3" s="22" t="n">
         <v>2.5</v>
       </c>
-      <c r="P3" s="23" t="n">
+      <c r="P3" s="22" t="n">
         <v>400</v>
       </c>
-      <c r="Q3" s="23" t="n">
+      <c r="Q3" s="22" t="n">
         <v>350</v>
       </c>
-      <c r="R3" s="23" t="n">
+      <c r="R3" s="22" t="n">
         <v>25</v>
       </c>
     </row>
@@ -4888,52 +4885,52 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="20" t="s">
         <v>216</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="22" t="s">
+      <c r="C2" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="D2" s="22" t="s">
+      <c r="D2" s="21" t="s">
         <v>193</v>
       </c>
-      <c r="E2" s="22" t="s">
+      <c r="E2" s="21" t="s">
         <v>238</v>
       </c>
-      <c r="F2" s="22" t="s">
+      <c r="F2" s="21" t="s">
         <v>239</v>
       </c>
-      <c r="G2" s="22" t="s">
+      <c r="G2" s="21" t="s">
         <v>240</v>
       </c>
-      <c r="H2" s="22" t="s">
+      <c r="H2" s="21" t="s">
         <v>241</v>
       </c>
-      <c r="I2" s="22" t="s">
+      <c r="I2" s="21" t="s">
         <v>242</v>
       </c>
-      <c r="J2" s="22" t="s">
+      <c r="J2" s="21" t="s">
         <v>243</v>
       </c>
-      <c r="K2" s="22" t="s">
+      <c r="K2" s="21" t="s">
         <v>244</v>
       </c>
       <c r="XFB2" s="3"/>
@@ -4941,110 +4938,110 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="22" t="s">
         <v>131</v>
       </c>
-      <c r="B3" s="23" t="s">
+      <c r="B3" s="22" t="s">
         <v>245</v>
       </c>
-      <c r="C3" s="23" t="s">
+      <c r="C3" s="22" t="s">
         <v>246</v>
       </c>
-      <c r="D3" s="23" t="s">
+      <c r="D3" s="22" t="s">
         <v>247</v>
       </c>
-      <c r="E3" s="23" t="s">
+      <c r="E3" s="22" t="s">
         <v>248</v>
       </c>
-      <c r="F3" s="23" t="s">
+      <c r="F3" s="22" t="s">
         <v>249</v>
       </c>
-      <c r="G3" s="24" t="b">
+      <c r="G3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H3" s="23" t="s">
+      <c r="H3" s="22" t="s">
         <v>250</v>
       </c>
-      <c r="I3" s="23" t="n">
+      <c r="I3" s="22" t="n">
         <v>0.5</v>
       </c>
-      <c r="J3" s="23" t="n">
+      <c r="J3" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="K3" s="23" t="n">
+      <c r="K3" s="22" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="22" t="s">
         <v>251</v>
       </c>
-      <c r="C4" s="23" t="s">
+      <c r="C4" s="22" t="s">
         <v>246</v>
       </c>
-      <c r="D4" s="23" t="s">
+      <c r="D4" s="22" t="s">
         <v>199</v>
       </c>
-      <c r="E4" s="23" t="s">
+      <c r="E4" s="22" t="s">
         <v>248</v>
       </c>
-      <c r="F4" s="23" t="s">
+      <c r="F4" s="22" t="s">
         <v>249</v>
       </c>
-      <c r="G4" s="24" t="b">
+      <c r="G4" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H4" s="23" t="s">
+      <c r="H4" s="22" t="s">
         <v>250</v>
       </c>
-      <c r="I4" s="23" t="n">
+      <c r="I4" s="22" t="n">
         <v>0.5</v>
       </c>
-      <c r="J4" s="23" t="n">
+      <c r="J4" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="K4" s="23" t="n">
+      <c r="K4" s="22" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="23" t="s">
+      <c r="A5" s="22" t="s">
         <v>168</v>
       </c>
-      <c r="B5" s="23" t="s">
+      <c r="B5" s="22" t="s">
         <v>252</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="C5" s="22" t="s">
         <v>246</v>
       </c>
-      <c r="D5" s="23" t="s">
+      <c r="D5" s="22" t="s">
         <v>253</v>
       </c>
-      <c r="E5" s="23" t="s">
+      <c r="E5" s="22" t="s">
         <v>248</v>
       </c>
-      <c r="F5" s="23" t="s">
+      <c r="F5" s="22" t="s">
         <v>254</v>
       </c>
-      <c r="G5" s="24" t="b">
+      <c r="G5" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H5" s="23" t="s">
+      <c r="H5" s="22" t="s">
         <v>255</v>
       </c>
-      <c r="I5" s="23" t="n">
+      <c r="I5" s="22" t="n">
         <v>0.5</v>
       </c>
-      <c r="J5" s="23" t="n">
+      <c r="J5" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="K5" s="23" t="n">
+      <c r="K5" s="22" t="n">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adjust central camera focal to enclose every cluster
</commit_message>
<xml_diff>
--- a/src/flychams_common/config/Configuration-Heterogeneous-Benchmark.xlsx
+++ b/src/flychams_common/config/Configuration-Heterogeneous-Benchmark.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="266">
   <si>
     <t xml:space="preserve">GENERAL CONFIGURATION</t>
   </si>
@@ -64,87 +64,87 @@
     <t xml:space="preserve">StartHour</t>
   </si>
   <si>
+    <t xml:space="preserve">MISSION00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Homogeneus Configuration (A) Dispersed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENVIRONMENT00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GROUP00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEAM00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(-200.0, 200.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(15.0, 150.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PX4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(13/12/2024)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(16:30:00)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MISSION01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Homogeneus Configuration (B) Dispersed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEAM01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MISSION02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Heterogeneus Configuration Dispersed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEAM02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MISSION03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Homogeneus Configuration (A) Concentrated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GROUP01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MISSION04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Homogeneus Configuration (B) Concentrated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MISSION05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Heterogeneus Configuration Concentrated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MISSION06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Homogeneus Configuration (A) Mixed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GROUP02</t>
+  </si>
+  <si>
     <t xml:space="preserve">X</t>
   </si>
   <si>
-    <t xml:space="preserve">MISSION00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Homogeneus Configuration (A) Dispersed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ENVIRONMENT00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GROUP00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TEAM00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(-200.0, 200.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(30.0, 150.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PX4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(13/12/2024)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(16:30:00)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MISSION01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Homogeneus Configuration (B) Dispersed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TEAM01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MISSION02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Heterogeneus Configuration Dispersed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TEAM02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MISSION03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Homogeneus Configuration (A) Concentrated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GROUP01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MISSION04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Homogeneus Configuration (B) Concentrated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MISSION05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Heterogeneus Configuration Concentrated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MISSION06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Homogeneus Configuration (A) Mixed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GROUP02</t>
-  </si>
-  <si>
     <t xml:space="preserve">MISSION07</t>
   </si>
   <si>
@@ -610,181 +610,181 @@
     <t xml:space="preserve">rtsp://127.0.0.1:8554/AGENT07/MULTICAMERA16</t>
   </si>
   <si>
+    <t xml:space="preserve">MinLambda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MaxLambda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RefLambda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MULTIWINDOW00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tracking Window 1.1 Multi-Window (2 Windows)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MULTIWINDOW01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tracking Window 1.2 Multi-Window (2 Windows)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MULTIWINDOW02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tracking Window 2.1 Multi-Window (2 Windows)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MULTIWINDOW03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tracking Window 2.2 Multi-Window (2 Windows)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MULTIWINDOW04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tracking Window 3.1 Multi-Window (2 Windows)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MULTIWINDOW05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tracking Window 3.2 Multi-Window (2 Windows)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MULTIWINDOW06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tracking Window 2.1 Multi-Window (3 Windows)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MULTIWINDOW07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tracking Window 2.2 Multi-Window (3 Windows)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MULTIWINDOW08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tracking Window 2.3 Multi-Window (3 Windows)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HARDWARE CATALOGS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CruiseSpeed [m/s]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MaxSpeed [m/s]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EnableBarometer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barometer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EnableIMU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EnableGPS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EnableMagnetometer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Magnetometer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BaseWeight [kg]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MaxPayloadWeight [kg]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HoverPower [W]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CruisePower [W]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LoadFactor [W/kg]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quadcopter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(WhiteNoiseSigma=8.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(AngularWhiteNoiseSigma=0.8, VelocityWhiteNoiseSigma=0.6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(EphIni=50, EpvIni=50, EphFin=2.0, EpvFin=2.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(WhiteNoiseSigma=0.02, WhiteNoiseBias=0)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resolution [pix]</t>
   </si>
   <si>
-    <t xml:space="preserve">MinLambda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MaxLambda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RefLambda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MULTIWINDOW00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tracking Window 1.1 Multi-Window (2 Windows)</t>
+    <t xml:space="preserve">SensorSize [mm]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distortion (K1, K2, K3, P1, P2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EnableSensorNoise</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SensorNoise</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weight [kg]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IdlePower [W]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ActivePower [W]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low-Resolution Central Camera</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RGB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(1280x720)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(13.2x7.425)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(-0.03, 0.002, 0.0, 0.0005, -0.0004)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(RandContrib=0.001, RandSize=100, RandSpeed=50000)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low-Resolution Tracking Camera</t>
   </si>
   <si>
     <t xml:space="preserve">(960x540)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MULTIWINDOW01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tracking Window 1.2 Multi-Window (2 Windows)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MULTIWINDOW02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tracking Window 2.1 Multi-Window (2 Windows)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MULTIWINDOW03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tracking Window 2.2 Multi-Window (2 Windows)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MULTIWINDOW04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tracking Window 3.1 Multi-Window (2 Windows)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MULTIWINDOW05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tracking Window 3.2 Multi-Window (2 Windows)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MULTIWINDOW06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tracking Window 2.1 Multi-Window (3 Windows)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MULTIWINDOW07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tracking Window 2.2 Multi-Window (3 Windows)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MULTIWINDOW08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tracking Window 2.3 Multi-Window (3 Windows)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HARDWARE CATALOGS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CruiseSpeed [m/s]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MaxSpeed [m/s]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EnableBarometer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Barometer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EnableIMU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IMU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EnableGPS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EnableMagnetometer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Magnetometer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BaseWeight [kg]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MaxPayloadWeight [kg]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HoverPower [W]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CruisePower [W]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LoadFactor [W/kg]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">x500</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quadcopter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(WhiteNoiseSigma=8.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(AngularWhiteNoiseSigma=0.8, VelocityWhiteNoiseSigma=0.6)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(EphIni=50, EpvIni=50, EphFin=2.0, EpvFin=2.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(WhiteNoiseSigma=0.02, WhiteNoiseBias=0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SensorSize [mm]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Distortion (K1, K2, K3, P1, P2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EnableSensorNoise</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SensorNoise</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weight [kg]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IdlePower [W]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ActivePower [W]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Low-Resolution Central Camera</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RGB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(1280x720)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(13.2x7.425)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(-0.03, 0.002, 0.0, 0.0005, -0.0004)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(RandContrib=0.001, RandSize=100, RandSpeed=50000)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Low-Resolution Tracking Camera</t>
   </si>
   <si>
     <t xml:space="preserve">High-Resolution Central Camera</t>
@@ -839,7 +839,7 @@
     <numFmt numFmtId="166" formatCode="0"/>
     <numFmt numFmtId="167" formatCode="General"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -900,13 +900,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="16"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -1007,7 +1000,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1040,7 +1033,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1052,16 +1045,12 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -1287,16 +1276,15 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table210_2" displayName="Table210_2" ref="A2:G4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A2:G4"/>
-  <tableColumns count="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table210_2" displayName="Table210_2" ref="A2:F4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A2:F4"/>
+  <tableColumns count="6">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Name"/>
     <tableColumn id="3" name="ObservationSetID"/>
-    <tableColumn id="4" name="Resolution [pix]"/>
-    <tableColumn id="5" name="MinLambda"/>
-    <tableColumn id="6" name="MaxLambda"/>
-    <tableColumn id="7" name="RefLambda"/>
+    <tableColumn id="4" name="MinLambda"/>
+    <tableColumn id="5" name="MaxLambda"/>
+    <tableColumn id="6" name="RefLambda"/>
   </tableColumns>
 </table>
 </file>
@@ -1649,38 +1637,36 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="8"/>
+      <c r="B3" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="C3" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="D3" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="E3" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="F3" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="G3" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="11" t="s">
+      <c r="H3" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="11" t="s">
+      <c r="I3" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I3" s="11" t="s">
+      <c r="J3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="K3" s="9" t="s">
         <v>20</v>
-      </c>
-      <c r="K3" s="9" t="s">
-        <v>21</v>
       </c>
       <c r="L3" s="12"/>
       <c r="M3" s="12"/>
@@ -1729,36 +1715,36 @@
       <c r="BD3" s="12"/>
     </row>
     <row r="4" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13"/>
+      <c r="A4" s="8"/>
       <c r="B4" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="D4" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>24</v>
-      </c>
       <c r="G4" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="H4" s="11" t="s">
+      <c r="I4" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I4" s="11" t="s">
+      <c r="J4" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="J4" s="9" t="s">
+      <c r="K4" s="9" t="s">
         <v>20</v>
-      </c>
-      <c r="K4" s="9" t="s">
-        <v>21</v>
       </c>
       <c r="L4" s="12"/>
       <c r="M4" s="12"/>
@@ -1807,36 +1793,36 @@
       <c r="BD4" s="12"/>
     </row>
     <row r="5" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13"/>
+      <c r="A5" s="8"/>
       <c r="B5" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="D5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" s="11" t="s">
-        <v>27</v>
-      </c>
       <c r="G5" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="11" t="s">
+      <c r="I5" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I5" s="11" t="s">
+      <c r="J5" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="J5" s="9" t="s">
+      <c r="K5" s="9" t="s">
         <v>20</v>
-      </c>
-      <c r="K5" s="9" t="s">
-        <v>21</v>
       </c>
       <c r="L5" s="12"/>
       <c r="M5" s="12"/>
@@ -1885,36 +1871,36 @@
       <c r="BD5" s="12"/>
     </row>
     <row r="6" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13"/>
+      <c r="A6" s="8"/>
       <c r="B6" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="D6" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>30</v>
-      </c>
       <c r="F6" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="H6" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="I6" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I6" s="11" t="s">
+      <c r="J6" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="J6" s="9" t="s">
+      <c r="K6" s="9" t="s">
         <v>20</v>
-      </c>
-      <c r="K6" s="9" t="s">
-        <v>21</v>
       </c>
       <c r="L6" s="12"/>
       <c r="M6" s="12"/>
@@ -1963,36 +1949,36 @@
       <c r="BD6" s="12"/>
     </row>
     <row r="7" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13"/>
+      <c r="A7" s="8"/>
       <c r="B7" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="10" t="s">
-        <v>32</v>
-      </c>
       <c r="D7" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G7" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="H7" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="11" t="s">
+      <c r="I7" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I7" s="11" t="s">
+      <c r="J7" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="J7" s="9" t="s">
+      <c r="K7" s="9" t="s">
         <v>20</v>
-      </c>
-      <c r="K7" s="9" t="s">
-        <v>21</v>
       </c>
       <c r="L7" s="12"/>
       <c r="M7" s="12"/>
@@ -2041,36 +2027,36 @@
       <c r="BD7" s="12"/>
     </row>
     <row r="8" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13"/>
+      <c r="A8" s="8"/>
       <c r="B8" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="10" t="s">
-        <v>34</v>
-      </c>
       <c r="D8" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G8" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="H8" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="H8" s="11" t="s">
+      <c r="I8" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I8" s="11" t="s">
+      <c r="J8" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="J8" s="9" t="s">
+      <c r="K8" s="9" t="s">
         <v>20</v>
-      </c>
-      <c r="K8" s="9" t="s">
-        <v>21</v>
       </c>
       <c r="L8" s="12"/>
       <c r="M8" s="12"/>
@@ -2119,36 +2105,36 @@
       <c r="BD8" s="12"/>
     </row>
     <row r="9" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13"/>
+      <c r="A9" s="8"/>
       <c r="B9" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="D9" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>37</v>
-      </c>
       <c r="F9" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="G9" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="H9" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="H9" s="11" t="s">
+      <c r="I9" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I9" s="11" t="s">
+      <c r="J9" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="J9" s="9" t="s">
+      <c r="K9" s="9" t="s">
         <v>20</v>
-      </c>
-      <c r="K9" s="9" t="s">
-        <v>21</v>
       </c>
       <c r="L9" s="12"/>
       <c r="M9" s="12"/>
@@ -2197,7 +2183,9 @@
       <c r="BD9" s="12"/>
     </row>
     <row r="10" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="13"/>
+      <c r="A10" s="8" t="s">
+        <v>37</v>
+      </c>
       <c r="B10" s="9" t="s">
         <v>38</v>
       </c>
@@ -2205,28 +2193,28 @@
         <v>39</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G10" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="H10" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="H10" s="11" t="s">
+      <c r="I10" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I10" s="11" t="s">
+      <c r="J10" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="J10" s="9" t="s">
+      <c r="K10" s="9" t="s">
         <v>20</v>
-      </c>
-      <c r="K10" s="9" t="s">
-        <v>21</v>
       </c>
       <c r="L10" s="12"/>
       <c r="M10" s="12"/>
@@ -2275,7 +2263,7 @@
       <c r="BD10" s="12"/>
     </row>
     <row r="11" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13"/>
+      <c r="A11" s="8"/>
       <c r="B11" s="9" t="s">
         <v>40</v>
       </c>
@@ -2283,28 +2271,28 @@
         <v>41</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G11" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="H11" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="H11" s="11" t="s">
+      <c r="I11" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I11" s="11" t="s">
+      <c r="J11" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="J11" s="9" t="s">
+      <c r="K11" s="9" t="s">
         <v>20</v>
-      </c>
-      <c r="K11" s="9" t="s">
-        <v>21</v>
       </c>
       <c r="L11" s="12"/>
       <c r="M11" s="12"/>
@@ -2389,92 +2377,92 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
-        <v>216</v>
-      </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
+      <c r="A1" s="19" t="s">
+        <v>214</v>
+      </c>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="20" t="s">
         <v>256</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="20" t="s">
         <v>257</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="20" t="s">
         <v>258</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="20" t="s">
         <v>259</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="20" t="s">
         <v>260</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="H2" s="20" t="s">
         <v>261</v>
       </c>
-      <c r="I2" s="21" t="s">
+      <c r="I2" s="20" t="s">
+        <v>241</v>
+      </c>
+      <c r="J2" s="20" t="s">
         <v>242</v>
       </c>
-      <c r="J2" s="21" t="s">
+      <c r="K2" s="20" t="s">
         <v>243</v>
-      </c>
-      <c r="K2" s="21" t="s">
-        <v>244</v>
       </c>
       <c r="L2" s="12"/>
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="21" t="s">
         <v>132</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="21" t="s">
         <v>262</v>
       </c>
-      <c r="C3" s="23" t="b">
+      <c r="C3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="21" t="s">
         <v>263</v>
       </c>
-      <c r="E3" s="23" t="b">
+      <c r="E3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="F3" s="22" t="s">
+      <c r="F3" s="21" t="s">
         <v>264</v>
       </c>
-      <c r="G3" s="23" t="b">
+      <c r="G3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H3" s="22" t="s">
+      <c r="H3" s="21" t="s">
         <v>265</v>
       </c>
-      <c r="I3" s="22" t="n">
+      <c r="I3" s="21" t="n">
         <v>0.4</v>
       </c>
-      <c r="J3" s="22" t="n">
+      <c r="J3" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="K3" s="22" t="n">
+      <c r="K3" s="21" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2528,12 +2516,12 @@
   </cols>
   <sheetData>
     <row r="1" s="7" customFormat="true" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
       <c r="E1" s="12"/>
       <c r="XFB1" s="3"/>
       <c r="XFC1" s="3"/>
@@ -2555,7 +2543,7 @@
     </row>
     <row r="3" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>44</v>
@@ -2563,7 +2551,7 @@
       <c r="C3" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="14" t="s">
         <v>46</v>
       </c>
     </row>
@@ -2577,7 +2565,7 @@
       <c r="C4" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="14" t="s">
         <v>49</v>
       </c>
     </row>
@@ -2617,15 +2605,15 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
     </row>
     <row r="2" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
@@ -2716,12 +2704,12 @@
         <v>55</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="E3" s="16" t="n">
+      <c r="E3" s="15" t="n">
         <v>16</v>
       </c>
       <c r="F3" s="9" t="s">
@@ -2797,12 +2785,12 @@
         <v>60</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D4" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="E4" s="16" t="n">
+      <c r="E4" s="15" t="n">
         <v>16</v>
       </c>
       <c r="F4" s="9" t="s">
@@ -2877,12 +2865,12 @@
         <v>63</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="E5" s="16" t="n">
+      <c r="E5" s="15" t="n">
         <v>16</v>
       </c>
       <c r="F5" s="9" t="s">
@@ -2997,48 +2985,48 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="H2" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="I2" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="J2" s="18" t="s">
+      <c r="J2" s="17" t="s">
         <v>72</v>
       </c>
       <c r="L2" s="12"/>
@@ -3053,258 +3041,258 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="C3" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="19" t="s">
+      <c r="C3" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H3" s="19" t="n">
+      <c r="H3" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I3" s="19" t="n">
+      <c r="I3" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J3" s="19" t="n">
+      <c r="J3" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="C4" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="19" t="s">
+      <c r="C4" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="E4" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="G4" s="19" t="s">
+      <c r="G4" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H4" s="19" t="n">
+      <c r="H4" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I4" s="19" t="n">
+      <c r="I4" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J4" s="19" t="n">
+      <c r="J4" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="C5" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" s="19" t="s">
+      <c r="C5" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="E5" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="F5" s="19" t="s">
+      <c r="F5" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="G5" s="19" t="s">
+      <c r="G5" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H5" s="19" t="n">
+      <c r="H5" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I5" s="19" t="n">
+      <c r="I5" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J5" s="19" t="n">
+      <c r="J5" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="C6" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" s="19" t="s">
+      <c r="C6" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E6" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="F6" s="19" t="s">
+      <c r="F6" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="G6" s="19" t="s">
+      <c r="G6" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H6" s="19" t="n">
+      <c r="H6" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I6" s="19" t="n">
+      <c r="I6" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J6" s="19" t="n">
+      <c r="J6" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="C7" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" s="19" t="s">
+      <c r="C7" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H7" s="19" t="n">
+      <c r="H7" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I7" s="19" t="n">
+      <c r="I7" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J7" s="19" t="n">
+      <c r="J7" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="C8" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" s="19" t="s">
+      <c r="C8" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="F8" s="19" t="s">
+      <c r="F8" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="G8" s="19" t="s">
+      <c r="G8" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H8" s="19" t="n">
+      <c r="H8" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I8" s="19" t="n">
+      <c r="I8" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J8" s="19" t="n">
+      <c r="J8" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="C9" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" s="19" t="s">
+      <c r="C9" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="F9" s="19" t="s">
+      <c r="F9" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="G9" s="19" t="s">
+      <c r="G9" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H9" s="19" t="n">
+      <c r="H9" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I9" s="19" t="n">
+      <c r="I9" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J9" s="19" t="n">
+      <c r="J9" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="18" t="s">
         <v>100</v>
       </c>
-      <c r="C10" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" s="19" t="s">
+      <c r="C10" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="E10" s="19" t="s">
+      <c r="E10" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="F10" s="19" t="s">
+      <c r="F10" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="G10" s="19" t="s">
+      <c r="G10" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="19" t="n">
+      <c r="H10" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I10" s="19" t="n">
+      <c r="I10" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J10" s="19" t="n">
+      <c r="J10" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
@@ -3350,32 +3338,32 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>105</v>
       </c>
       <c r="H2" s="12"/>
@@ -3391,23 +3379,23 @@
       <c r="XFD2" s="12"/>
     </row>
     <row r="3" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="D3" s="19" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E3" s="19" t="n">
+      <c r="D3" s="18" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E3" s="18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F3" s="18" t="n">
         <v>0.9</v>
-      </c>
-      <c r="F3" s="19" t="n">
-        <v>0.8</v>
       </c>
       <c r="G3" s="2"/>
       <c r="XEV3" s="2"/>
@@ -3416,23 +3404,23 @@
       <c r="XEY3" s="3"/>
     </row>
     <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="D4" s="19" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E4" s="19" t="n">
+      <c r="D4" s="18" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E4" s="18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F4" s="18" t="n">
         <v>0.9</v>
-      </c>
-      <c r="F4" s="19" t="n">
-        <v>0.8</v>
       </c>
       <c r="G4" s="2"/>
       <c r="XEV4" s="2"/>
@@ -3441,23 +3429,23 @@
       <c r="XEY4" s="3"/>
     </row>
     <row r="5" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D5" s="19" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E5" s="19" t="n">
+      <c r="D5" s="18" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E5" s="18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F5" s="18" t="n">
         <v>0.9</v>
-      </c>
-      <c r="F5" s="19" t="n">
-        <v>0.8</v>
       </c>
       <c r="G5" s="2"/>
       <c r="XEV5" s="2"/>
@@ -3466,23 +3454,23 @@
       <c r="XEY5" s="3"/>
     </row>
     <row r="6" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="D6" s="19" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E6" s="19" t="n">
+      <c r="D6" s="18" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E6" s="18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F6" s="18" t="n">
         <v>0.9</v>
-      </c>
-      <c r="F6" s="19" t="n">
-        <v>0.8</v>
       </c>
       <c r="G6" s="2"/>
       <c r="XEV6" s="2"/>
@@ -3491,23 +3479,23 @@
       <c r="XEY6" s="3"/>
     </row>
     <row r="7" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="D7" s="19" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E7" s="19" t="n">
+      <c r="D7" s="18" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E7" s="18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F7" s="18" t="n">
         <v>0.9</v>
-      </c>
-      <c r="F7" s="19" t="n">
-        <v>0.8</v>
       </c>
       <c r="G7" s="2"/>
       <c r="XEV7" s="2"/>
@@ -3516,23 +3504,23 @@
       <c r="XEY7" s="3"/>
     </row>
     <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>116</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="D8" s="19" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E8" s="19" t="n">
+      <c r="D8" s="18" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E8" s="18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F8" s="18" t="n">
         <v>0.9</v>
-      </c>
-      <c r="F8" s="19" t="n">
-        <v>0.8</v>
       </c>
       <c r="G8" s="2"/>
       <c r="XEV8" s="2"/>
@@ -3541,23 +3529,23 @@
       <c r="XEY8" s="3"/>
     </row>
     <row r="9" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="18" t="s">
         <v>118</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D9" s="19" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E9" s="19" t="n">
+      <c r="D9" s="18" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E9" s="18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F9" s="18" t="n">
         <v>0.9</v>
-      </c>
-      <c r="F9" s="19" t="n">
-        <v>0.8</v>
       </c>
       <c r="G9" s="2"/>
       <c r="XEV9" s="2"/>
@@ -3566,23 +3554,23 @@
       <c r="XEY9" s="3"/>
     </row>
     <row r="10" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="D10" s="19" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E10" s="19" t="n">
+      <c r="D10" s="18" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E10" s="18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F10" s="18" t="n">
         <v>0.9</v>
-      </c>
-      <c r="F10" s="19" t="n">
-        <v>0.8</v>
       </c>
       <c r="G10" s="2"/>
       <c r="XEV10" s="2"/>
@@ -3647,56 +3635,56 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
-      <c r="L1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>124</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="H2" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="I2" s="17" t="s">
         <v>125</v>
       </c>
-      <c r="J2" s="18" t="s">
+      <c r="J2" s="17" t="s">
         <v>126</v>
       </c>
-      <c r="K2" s="18" t="s">
+      <c r="K2" s="17" t="s">
         <v>127</v>
       </c>
-      <c r="L2" s="18" t="s">
+      <c r="L2" s="17" t="s">
         <v>128</v>
       </c>
       <c r="M2" s="12"/>
@@ -3709,652 +3697,652 @@
       <c r="XFC2" s="12"/>
     </row>
     <row r="3" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>129</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>130</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="H3" s="19" t="s">
+      <c r="H3" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="I3" s="19" t="n">
+      <c r="I3" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="K3" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J3" s="19" t="n">
+      <c r="L3" s="18" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="18" t="s">
+        <v>137</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="E4" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="F4" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="G4" s="18" t="s">
+        <v>141</v>
+      </c>
+      <c r="H4" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="I4" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="18" t="n">
+        <v>40</v>
+      </c>
+      <c r="K4" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="L4" s="18" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="18" t="s">
+        <v>144</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>145</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="E5" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="F5" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="G5" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="H5" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="I5" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" s="18" t="n">
+        <v>40</v>
+      </c>
+      <c r="K5" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="L5" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="XFD5" s="12"/>
+    </row>
+    <row r="6" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>109</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>131</v>
+      </c>
+      <c r="E6" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="F6" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="G6" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="H6" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="I6" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="K6" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K3" s="19" t="n">
+      <c r="L6" s="18" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="7" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>109</v>
+      </c>
+      <c r="D7" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="E7" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="F7" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="G7" s="18" t="s">
+        <v>141</v>
+      </c>
+      <c r="H7" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="I7" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="18" t="n">
+        <v>40</v>
+      </c>
+      <c r="K7" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="L7" s="18" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="18" t="s">
+        <v>154</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>155</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>109</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="E8" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="F8" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="G8" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="H8" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="I8" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="18" t="n">
+        <v>40</v>
+      </c>
+      <c r="K8" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="L8" s="18" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="9" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="18" t="s">
+        <v>157</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>158</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="D9" s="18" t="s">
+        <v>131</v>
+      </c>
+      <c r="E9" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="F9" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="G9" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="H9" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="I9" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="K9" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L3" s="19" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
-        <v>137</v>
-      </c>
-      <c r="B4" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="C4" s="19" t="s">
-        <v>107</v>
-      </c>
-      <c r="D4" s="19" t="s">
+      <c r="L9" s="18" t="s">
+        <v>159</v>
+      </c>
+      <c r="XFD9" s="2"/>
+    </row>
+    <row r="10" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="18" t="s">
+        <v>160</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>161</v>
+      </c>
+      <c r="C10" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="D10" s="18" t="s">
         <v>139</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="E10" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F10" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="G4" s="19" t="s">
+      <c r="G10" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="H4" s="19" t="s">
+      <c r="H10" s="18" t="s">
         <v>142</v>
       </c>
-      <c r="I4" s="19" t="n">
+      <c r="I10" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="J4" s="19" t="n">
+      <c r="J10" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K4" s="19" t="n">
+      <c r="K10" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L4" s="19" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
-        <v>144</v>
-      </c>
-      <c r="B5" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="C5" s="19" t="s">
-        <v>107</v>
-      </c>
-      <c r="D5" s="19" t="s">
+      <c r="L10" s="18" t="s">
+        <v>162</v>
+      </c>
+      <c r="XFD10" s="2"/>
+    </row>
+    <row r="11" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>164</v>
+      </c>
+      <c r="C11" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="D11" s="18" t="s">
         <v>139</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="E11" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="F5" s="19" t="s">
+      <c r="F11" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="G5" s="19" t="s">
+      <c r="G11" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="H5" s="19" t="s">
+      <c r="H11" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="I5" s="19" t="n">
+      <c r="I11" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="J5" s="19" t="n">
+      <c r="J11" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K5" s="19" t="n">
+      <c r="K11" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L5" s="19" t="s">
-        <v>147</v>
-      </c>
-      <c r="XFD5" s="12"/>
-    </row>
-    <row r="6" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
-        <v>148</v>
-      </c>
-      <c r="B6" s="19" t="s">
-        <v>149</v>
-      </c>
-      <c r="C6" s="19" t="s">
-        <v>109</v>
-      </c>
-      <c r="D6" s="19" t="s">
+      <c r="L11" s="18" t="s">
+        <v>165</v>
+      </c>
+      <c r="XFD11" s="2"/>
+    </row>
+    <row r="12" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="18" t="s">
+        <v>166</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="E12" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="F12" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="G12" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="H12" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="I12" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="K12" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="L12" s="18" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>171</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="D13" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="E13" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="F13" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="G13" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="H13" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="I13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="K13" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="L13" s="18" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="18" t="s">
+        <v>173</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>174</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="E14" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="F14" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="G14" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="H14" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="I14" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="K14" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="L14" s="18" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="18" t="s">
+        <v>176</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>177</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="D15" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E15" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="F6" s="19" t="s">
+      <c r="F15" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="G6" s="19" t="s">
+      <c r="G15" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="H6" s="19" t="s">
+      <c r="H15" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="I6" s="19" t="n">
+      <c r="I15" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J15" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="K15" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J6" s="19" t="n">
+      <c r="L15" s="18" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>180</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="E16" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="F16" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="G16" s="18" t="s">
+        <v>141</v>
+      </c>
+      <c r="H16" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="I16" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" s="18" t="n">
+        <v>40</v>
+      </c>
+      <c r="K16" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="L16" s="18" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="18" t="s">
+        <v>182</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>183</v>
+      </c>
+      <c r="C17" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="E17" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="F17" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="G17" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="H17" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="I17" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" s="18" t="n">
+        <v>40</v>
+      </c>
+      <c r="K17" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="L17" s="18" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="18" t="s">
+        <v>185</v>
+      </c>
+      <c r="B18" s="18" t="s">
+        <v>186</v>
+      </c>
+      <c r="C18" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="D18" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="E18" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="F18" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="G18" s="18" t="s">
+        <v>187</v>
+      </c>
+      <c r="H18" s="18" t="s">
+        <v>188</v>
+      </c>
+      <c r="I18" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="18" t="n">
+        <v>40</v>
+      </c>
+      <c r="K18" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="L18" s="18" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="18" t="s">
+        <v>190</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>191</v>
+      </c>
+      <c r="C19" s="18" t="s">
+        <v>121</v>
+      </c>
+      <c r="D19" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="E19" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="F19" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="G19" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="H19" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="I19" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="K19" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K6" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="L6" s="19" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="7" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
-        <v>151</v>
-      </c>
-      <c r="B7" s="19" t="s">
-        <v>152</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>109</v>
-      </c>
-      <c r="D7" s="19" t="s">
-        <v>139</v>
-      </c>
-      <c r="E7" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="F7" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="G7" s="19" t="s">
-        <v>141</v>
-      </c>
-      <c r="H7" s="19" t="s">
-        <v>142</v>
-      </c>
-      <c r="I7" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" s="19" t="n">
-        <v>40</v>
-      </c>
-      <c r="K7" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="L7" s="19" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
-        <v>154</v>
-      </c>
-      <c r="B8" s="19" t="s">
-        <v>155</v>
-      </c>
-      <c r="C8" s="19" t="s">
-        <v>109</v>
-      </c>
-      <c r="D8" s="19" t="s">
-        <v>139</v>
-      </c>
-      <c r="E8" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="F8" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="G8" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="H8" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="I8" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="J8" s="19" t="n">
-        <v>40</v>
-      </c>
-      <c r="K8" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="L8" s="19" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="9" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
-        <v>157</v>
-      </c>
-      <c r="B9" s="19" t="s">
-        <v>158</v>
-      </c>
-      <c r="C9" s="19" t="s">
-        <v>111</v>
-      </c>
-      <c r="D9" s="19" t="s">
-        <v>131</v>
-      </c>
-      <c r="E9" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="F9" s="19" t="s">
-        <v>133</v>
-      </c>
-      <c r="G9" s="19" t="s">
-        <v>134</v>
-      </c>
-      <c r="H9" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="I9" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="J9" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="K9" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="L9" s="19" t="s">
-        <v>159</v>
-      </c>
-      <c r="XFD9" s="2"/>
-    </row>
-    <row r="10" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
-        <v>160</v>
-      </c>
-      <c r="B10" s="19" t="s">
-        <v>161</v>
-      </c>
-      <c r="C10" s="19" t="s">
-        <v>111</v>
-      </c>
-      <c r="D10" s="19" t="s">
-        <v>139</v>
-      </c>
-      <c r="E10" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="F10" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="G10" s="19" t="s">
-        <v>141</v>
-      </c>
-      <c r="H10" s="19" t="s">
-        <v>142</v>
-      </c>
-      <c r="I10" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="J10" s="19" t="n">
-        <v>40</v>
-      </c>
-      <c r="K10" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="L10" s="19" t="s">
-        <v>162</v>
-      </c>
-      <c r="XFD10" s="2"/>
-    </row>
-    <row r="11" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
-        <v>163</v>
-      </c>
-      <c r="B11" s="19" t="s">
-        <v>164</v>
-      </c>
-      <c r="C11" s="19" t="s">
-        <v>111</v>
-      </c>
-      <c r="D11" s="19" t="s">
-        <v>139</v>
-      </c>
-      <c r="E11" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="F11" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="G11" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="H11" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="I11" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="J11" s="19" t="n">
-        <v>40</v>
-      </c>
-      <c r="K11" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="L11" s="19" t="s">
-        <v>165</v>
-      </c>
-      <c r="XFD11" s="2"/>
-    </row>
-    <row r="12" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="19" t="s">
-        <v>166</v>
-      </c>
-      <c r="B12" s="19" t="s">
-        <v>167</v>
-      </c>
-      <c r="C12" s="19" t="s">
-        <v>113</v>
-      </c>
-      <c r="D12" s="19" t="s">
-        <v>168</v>
-      </c>
-      <c r="E12" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="F12" s="19" t="s">
-        <v>133</v>
-      </c>
-      <c r="G12" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="H12" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="I12" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="J12" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="K12" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="L12" s="19" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
-        <v>170</v>
-      </c>
-      <c r="B13" s="19" t="s">
-        <v>171</v>
-      </c>
-      <c r="C13" s="19" t="s">
-        <v>115</v>
-      </c>
-      <c r="D13" s="19" t="s">
-        <v>168</v>
-      </c>
-      <c r="E13" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="F13" s="19" t="s">
-        <v>133</v>
-      </c>
-      <c r="G13" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="H13" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="J13" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="K13" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="L13" s="19" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="19" t="s">
-        <v>173</v>
-      </c>
-      <c r="B14" s="19" t="s">
-        <v>174</v>
-      </c>
-      <c r="C14" s="19" t="s">
-        <v>117</v>
-      </c>
-      <c r="D14" s="19" t="s">
-        <v>168</v>
-      </c>
-      <c r="E14" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="F14" s="19" t="s">
-        <v>133</v>
-      </c>
-      <c r="G14" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="H14" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="I14" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="J14" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="K14" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="L14" s="19" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="19" t="s">
-        <v>176</v>
-      </c>
-      <c r="B15" s="19" t="s">
-        <v>177</v>
-      </c>
-      <c r="C15" s="19" t="s">
-        <v>119</v>
-      </c>
-      <c r="D15" s="19" t="s">
-        <v>131</v>
-      </c>
-      <c r="E15" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="F15" s="19" t="s">
-        <v>133</v>
-      </c>
-      <c r="G15" s="19" t="s">
-        <v>134</v>
-      </c>
-      <c r="H15" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="I15" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="J15" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="K15" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="L15" s="19" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="19" t="s">
-        <v>179</v>
-      </c>
-      <c r="B16" s="19" t="s">
-        <v>180</v>
-      </c>
-      <c r="C16" s="19" t="s">
-        <v>119</v>
-      </c>
-      <c r="D16" s="19" t="s">
-        <v>139</v>
-      </c>
-      <c r="E16" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="F16" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="G16" s="19" t="s">
-        <v>141</v>
-      </c>
-      <c r="H16" s="19" t="s">
-        <v>142</v>
-      </c>
-      <c r="I16" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="J16" s="19" t="n">
-        <v>40</v>
-      </c>
-      <c r="K16" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="L16" s="19" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="19" t="s">
-        <v>182</v>
-      </c>
-      <c r="B17" s="19" t="s">
-        <v>183</v>
-      </c>
-      <c r="C17" s="19" t="s">
-        <v>119</v>
-      </c>
-      <c r="D17" s="19" t="s">
-        <v>139</v>
-      </c>
-      <c r="E17" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="F17" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="G17" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="H17" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="I17" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="J17" s="19" t="n">
-        <v>40</v>
-      </c>
-      <c r="K17" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="L17" s="19" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="19" t="s">
-        <v>185</v>
-      </c>
-      <c r="B18" s="19" t="s">
-        <v>186</v>
-      </c>
-      <c r="C18" s="19" t="s">
-        <v>119</v>
-      </c>
-      <c r="D18" s="19" t="s">
-        <v>139</v>
-      </c>
-      <c r="E18" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="F18" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="G18" s="19" t="s">
-        <v>187</v>
-      </c>
-      <c r="H18" s="19" t="s">
-        <v>188</v>
-      </c>
-      <c r="I18" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="J18" s="19" t="n">
-        <v>40</v>
-      </c>
-      <c r="K18" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="L18" s="19" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="19" t="s">
-        <v>190</v>
-      </c>
-      <c r="B19" s="19" t="s">
-        <v>191</v>
-      </c>
-      <c r="C19" s="19" t="s">
-        <v>121</v>
-      </c>
-      <c r="D19" s="19" t="s">
-        <v>168</v>
-      </c>
-      <c r="E19" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="F19" s="19" t="s">
-        <v>133</v>
-      </c>
-      <c r="G19" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="H19" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="I19" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="J19" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="K19" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="L19" s="19" t="s">
+      <c r="L19" s="18" t="s">
         <v>192</v>
       </c>
     </row>
@@ -4385,48 +4373,44 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="27.35"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="57.21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="27.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="12" width="27.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="2" width="27.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="12" width="27.35"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16374" min="8" style="2" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16383" min="16375" style="3" width="10.49"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="3" width="10.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="2" width="27.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="12" width="27.35"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16373" min="7" style="2" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16382" min="16374" style="3" width="10.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16383" min="16383" style="0" width="10.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="3" width="9.34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>193</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>194</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>195</v>
       </c>
-      <c r="G2" s="18" t="s">
-        <v>196</v>
-      </c>
+      <c r="XET2" s="3"/>
       <c r="XEU2" s="3"/>
       <c r="XEV2" s="3"/>
       <c r="XEW2" s="3"/>
@@ -4435,214 +4419,187 @@
       <c r="XEZ2" s="3"/>
       <c r="XFA2" s="3"/>
       <c r="XFB2" s="3"/>
-      <c r="XFC2" s="3"/>
+      <c r="XFC2" s="0"/>
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
+        <v>196</v>
+      </c>
+      <c r="B3" s="18" t="s">
         <v>197</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="C3" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="D3" s="18" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E3" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="18" t="n">
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="18" t="s">
         <v>198</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="B4" s="18" t="s">
+        <v>199</v>
+      </c>
+      <c r="C4" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="D3" s="19" t="s">
-        <v>199</v>
-      </c>
-      <c r="E3" s="19" t="n">
-        <v>0.167</v>
-      </c>
-      <c r="F3" s="19" t="n">
+      <c r="D4" s="18" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E4" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G3" s="19" t="n">
-        <v>0.583</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="F4" s="18" t="n">
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="18" t="s">
         <v>200</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B5" s="18" t="s">
         <v>201</v>
       </c>
-      <c r="C4" s="19" t="s">
-        <v>113</v>
-      </c>
-      <c r="D4" s="19" t="s">
-        <v>199</v>
-      </c>
-      <c r="E4" s="19" t="n">
-        <v>0.167</v>
-      </c>
-      <c r="F4" s="19" t="n">
+      <c r="C5" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="D5" s="18" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E5" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="19" t="n">
-        <v>0.583</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="F5" s="18" t="n">
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="18" t="s">
         <v>202</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>203</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C6" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="D5" s="19" t="s">
-        <v>199</v>
-      </c>
-      <c r="E5" s="19" t="n">
-        <v>0.167</v>
-      </c>
-      <c r="F5" s="19" t="n">
+      <c r="D6" s="18" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E6" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G5" s="19" t="n">
-        <v>0.583</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+      <c r="F6" s="18" t="n">
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>205</v>
       </c>
-      <c r="C6" s="19" t="s">
-        <v>115</v>
-      </c>
-      <c r="D6" s="19" t="s">
-        <v>199</v>
-      </c>
-      <c r="E6" s="19" t="n">
-        <v>0.167</v>
-      </c>
-      <c r="F6" s="19" t="n">
+      <c r="C7" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="D7" s="18" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E7" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G6" s="19" t="n">
-        <v>0.583</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+      <c r="F7" s="18" t="n">
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="18" t="s">
         <v>206</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>207</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C8" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="D7" s="19" t="s">
-        <v>199</v>
-      </c>
-      <c r="E7" s="19" t="n">
-        <v>0.167</v>
-      </c>
-      <c r="F7" s="19" t="n">
+      <c r="D8" s="18" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E8" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="19" t="n">
-        <v>0.583</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="F8" s="18" t="n">
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="18" t="s">
         <v>208</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B9" s="18" t="s">
         <v>209</v>
       </c>
-      <c r="C8" s="19" t="s">
-        <v>117</v>
-      </c>
-      <c r="D8" s="19" t="s">
-        <v>199</v>
-      </c>
-      <c r="E8" s="19" t="n">
-        <v>0.167</v>
-      </c>
-      <c r="F8" s="19" t="n">
+      <c r="C9" s="18" t="s">
+        <v>121</v>
+      </c>
+      <c r="D9" s="18" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E9" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="19" t="n">
-        <v>0.583</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
+      <c r="F9" s="18" t="n">
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="18" t="s">
         <v>210</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B10" s="18" t="s">
         <v>211</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C10" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="D9" s="19" t="s">
-        <v>199</v>
-      </c>
-      <c r="E9" s="19" t="n">
-        <v>0.167</v>
-      </c>
-      <c r="F9" s="19" t="n">
+      <c r="D10" s="18" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E10" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="19" t="n">
-        <v>0.583</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+      <c r="F10" s="18" t="n">
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="18" t="s">
         <v>212</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B11" s="18" t="s">
         <v>213</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C11" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="D10" s="19" t="s">
-        <v>199</v>
-      </c>
-      <c r="E10" s="19" t="n">
-        <v>0.167</v>
-      </c>
-      <c r="F10" s="19" t="n">
+      <c r="D11" s="18" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E11" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="19" t="n">
-        <v>0.583</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
-        <v>214</v>
-      </c>
-      <c r="B11" s="19" t="s">
-        <v>215</v>
-      </c>
-      <c r="C11" s="19" t="s">
-        <v>121</v>
-      </c>
-      <c r="D11" s="19" t="s">
-        <v>199</v>
-      </c>
-      <c r="E11" s="19" t="n">
-        <v>0.167</v>
-      </c>
-      <c r="F11" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" s="19" t="n">
-        <v>0.583</v>
+      <c r="F11" s="18" t="n">
+        <v>0.625</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -4653,7 +4610,7 @@
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4692,140 +4649,140 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="19" t="s">
+        <v>214</v>
+      </c>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
+      <c r="O1" s="19"/>
+      <c r="P1" s="19"/>
+      <c r="Q1" s="19"/>
+      <c r="R1" s="19"/>
+    </row>
+    <row r="2" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="D2" s="20" t="s">
+        <v>215</v>
+      </c>
+      <c r="E2" s="20" t="s">
         <v>216</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
-      <c r="O1" s="20"/>
-      <c r="P1" s="20"/>
-      <c r="Q1" s="20"/>
-      <c r="R1" s="20"/>
-    </row>
-    <row r="2" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="21" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="21" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="D2" s="21" t="s">
+      <c r="F2" s="20" t="s">
         <v>217</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="G2" s="20" t="s">
         <v>218</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="H2" s="20" t="s">
         <v>219</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="I2" s="20" t="s">
         <v>220</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="J2" s="20" t="s">
         <v>221</v>
       </c>
-      <c r="I2" s="21" t="s">
+      <c r="K2" s="20" t="s">
         <v>222</v>
       </c>
-      <c r="J2" s="21" t="s">
+      <c r="L2" s="20" t="s">
         <v>223</v>
       </c>
-      <c r="K2" s="21" t="s">
+      <c r="M2" s="20" t="s">
         <v>224</v>
       </c>
-      <c r="L2" s="21" t="s">
+      <c r="N2" s="20" t="s">
         <v>225</v>
       </c>
-      <c r="M2" s="21" t="s">
+      <c r="O2" s="20" t="s">
         <v>226</v>
       </c>
-      <c r="N2" s="21" t="s">
+      <c r="P2" s="20" t="s">
         <v>227</v>
       </c>
-      <c r="O2" s="21" t="s">
+      <c r="Q2" s="20" t="s">
         <v>228</v>
       </c>
-      <c r="P2" s="21" t="s">
+      <c r="R2" s="20" t="s">
         <v>229</v>
       </c>
-      <c r="Q2" s="21" t="s">
+    </row>
+    <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="B3" s="21" t="s">
         <v>230</v>
       </c>
-      <c r="R2" s="21" t="s">
+      <c r="C3" s="21" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="22" t="s">
-        <v>76</v>
-      </c>
-      <c r="B3" s="22" t="s">
-        <v>232</v>
-      </c>
-      <c r="C3" s="22" t="s">
-        <v>233</v>
-      </c>
-      <c r="D3" s="22" t="n">
+      <c r="D3" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="E3" s="22" t="n">
+      <c r="E3" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="F3" s="23" t="b">
+      <c r="F3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="G3" s="22" t="s">
-        <v>234</v>
-      </c>
-      <c r="H3" s="23" t="b">
+      <c r="G3" s="21" t="s">
+        <v>232</v>
+      </c>
+      <c r="H3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="I3" s="22" t="s">
-        <v>235</v>
-      </c>
-      <c r="J3" s="23" t="b">
+      <c r="I3" s="21" t="s">
+        <v>233</v>
+      </c>
+      <c r="J3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="K3" s="22" t="s">
-        <v>236</v>
-      </c>
-      <c r="L3" s="23" t="b">
+      <c r="K3" s="21" t="s">
+        <v>234</v>
+      </c>
+      <c r="L3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="M3" s="22" t="s">
-        <v>237</v>
-      </c>
-      <c r="N3" s="22" t="n">
+      <c r="M3" s="21" t="s">
+        <v>235</v>
+      </c>
+      <c r="N3" s="21" t="n">
         <v>6.5</v>
       </c>
-      <c r="O3" s="22" t="n">
+      <c r="O3" s="21" t="n">
         <v>2.5</v>
       </c>
-      <c r="P3" s="22" t="n">
+      <c r="P3" s="21" t="n">
         <v>400</v>
       </c>
-      <c r="Q3" s="22" t="n">
+      <c r="Q3" s="21" t="n">
         <v>350</v>
       </c>
-      <c r="R3" s="22" t="n">
+      <c r="R3" s="21" t="n">
         <v>25</v>
       </c>
     </row>
@@ -4885,163 +4842,163 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
-        <v>216</v>
-      </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
+      <c r="A1" s="19" t="s">
+        <v>214</v>
+      </c>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="D2" s="21" t="s">
-        <v>193</v>
-      </c>
-      <c r="E2" s="21" t="s">
+      <c r="D2" s="20" t="s">
+        <v>236</v>
+      </c>
+      <c r="E2" s="20" t="s">
+        <v>237</v>
+      </c>
+      <c r="F2" s="20" t="s">
         <v>238</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="G2" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="H2" s="20" t="s">
         <v>240</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="I2" s="20" t="s">
         <v>241</v>
       </c>
-      <c r="I2" s="21" t="s">
+      <c r="J2" s="20" t="s">
         <v>242</v>
       </c>
-      <c r="J2" s="21" t="s">
+      <c r="K2" s="20" t="s">
         <v>243</v>
-      </c>
-      <c r="K2" s="21" t="s">
-        <v>244</v>
       </c>
       <c r="XFB2" s="3"/>
       <c r="XFC2" s="3"/>
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="21" t="s">
         <v>131</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="21" t="s">
+        <v>244</v>
+      </c>
+      <c r="C3" s="21" t="s">
         <v>245</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="D3" s="21" t="s">
         <v>246</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="E3" s="21" t="s">
         <v>247</v>
       </c>
-      <c r="E3" s="22" t="s">
+      <c r="F3" s="21" t="s">
         <v>248</v>
       </c>
-      <c r="F3" s="22" t="s">
-        <v>249</v>
-      </c>
-      <c r="G3" s="23" t="b">
+      <c r="G3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H3" s="22" t="s">
+      <c r="H3" s="21" t="s">
+        <v>249</v>
+      </c>
+      <c r="I3" s="21" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J3" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="K3" s="21" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="21" t="s">
+        <v>139</v>
+      </c>
+      <c r="B4" s="21" t="s">
         <v>250</v>
       </c>
-      <c r="I3" s="22" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="J3" s="22" t="n">
-        <v>2</v>
-      </c>
-      <c r="K3" s="22" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="22" t="s">
-        <v>139</v>
-      </c>
-      <c r="B4" s="22" t="s">
+      <c r="C4" s="21" t="s">
+        <v>245</v>
+      </c>
+      <c r="D4" s="21" t="s">
         <v>251</v>
       </c>
-      <c r="C4" s="22" t="s">
-        <v>246</v>
-      </c>
-      <c r="D4" s="22" t="s">
-        <v>199</v>
-      </c>
-      <c r="E4" s="22" t="s">
+      <c r="E4" s="21" t="s">
+        <v>247</v>
+      </c>
+      <c r="F4" s="21" t="s">
         <v>248</v>
       </c>
-      <c r="F4" s="22" t="s">
-        <v>249</v>
-      </c>
-      <c r="G4" s="23" t="b">
+      <c r="G4" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H4" s="22" t="s">
-        <v>250</v>
-      </c>
-      <c r="I4" s="22" t="n">
+      <c r="H4" s="21" t="s">
+        <v>249</v>
+      </c>
+      <c r="I4" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="J4" s="22" t="n">
+      <c r="J4" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="K4" s="22" t="n">
+      <c r="K4" s="21" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="21" t="s">
         <v>168</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="21" t="s">
         <v>252</v>
       </c>
-      <c r="C5" s="22" t="s">
-        <v>246</v>
-      </c>
-      <c r="D5" s="22" t="s">
+      <c r="C5" s="21" t="s">
+        <v>245</v>
+      </c>
+      <c r="D5" s="21" t="s">
         <v>253</v>
       </c>
-      <c r="E5" s="22" t="s">
-        <v>248</v>
-      </c>
-      <c r="F5" s="22" t="s">
+      <c r="E5" s="21" t="s">
+        <v>247</v>
+      </c>
+      <c r="F5" s="21" t="s">
         <v>254</v>
       </c>
-      <c r="G5" s="23" t="b">
+      <c r="G5" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H5" s="22" t="s">
+      <c r="H5" s="21" t="s">
         <v>255</v>
       </c>
-      <c r="I5" s="22" t="n">
+      <c r="I5" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="J5" s="22" t="n">
+      <c r="J5" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="K5" s="22" t="n">
+      <c r="K5" s="21" t="n">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve cluster trajectories setups
</commit_message>
<xml_diff>
--- a/src/flychams_common/config/Configuration-Heterogeneous-Benchmark.xlsx
+++ b/src/flychams_common/config/Configuration-Heterogeneous-Benchmark.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Mission" sheetId="1" state="visible" r:id="rId3"/>
@@ -142,15 +142,15 @@
     <t xml:space="preserve">GROUP02</t>
   </si>
   <si>
+    <t xml:space="preserve">MISSION07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Homogeneus Configuration (B) Mixed</t>
+  </si>
+  <si>
     <t xml:space="preserve">X</t>
   </si>
   <si>
-    <t xml:space="preserve">MISSION07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Homogeneus Configuration (B) Mixed</t>
-  </si>
-  <si>
     <t xml:space="preserve">MISSION08</t>
   </si>
   <si>
@@ -205,25 +205,7 @@
     <t xml:space="preserve">High</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Complex-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Dispersed</t>
-    </r>
+    <t xml:space="preserve">Complex-Dispersed</t>
   </si>
   <si>
     <t xml:space="preserve">TARGET01</t>
@@ -232,25 +214,7 @@
     <t xml:space="preserve">Concentrated Configuration (6 Clusters)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Complex-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Concentrated</t>
-    </r>
+    <t xml:space="preserve">Complex-Concentrated</t>
   </si>
   <si>
     <t xml:space="preserve">TARGET02</t>
@@ -945,8 +909,9 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
+      <b val="true"/>
+      <sz val="16"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -1095,6 +1060,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1107,11 +1076,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2155,7 +2120,7 @@
       <c r="BD8" s="12"/>
     </row>
     <row r="9" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8"/>
+      <c r="A9" s="13"/>
       <c r="B9" s="9" t="s">
         <v>34</v>
       </c>
@@ -2233,14 +2198,12 @@
       <c r="BD9" s="12"/>
     </row>
     <row r="10" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="13"/>
+      <c r="B10" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="C10" s="10" t="s">
         <v>38</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>39</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>13</v>
@@ -2313,7 +2276,9 @@
       <c r="BD10" s="12"/>
     </row>
     <row r="11" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8"/>
+      <c r="A11" s="13" t="s">
+        <v>39</v>
+      </c>
       <c r="B11" s="9" t="s">
         <v>40</v>
       </c>
@@ -2566,12 +2531,12 @@
   </cols>
   <sheetData>
     <row r="1" s="7" customFormat="true" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
       <c r="E1" s="12"/>
       <c r="XFB1" s="3"/>
       <c r="XFC1" s="3"/>
@@ -2601,7 +2566,7 @@
       <c r="C3" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="15" t="s">
         <v>46</v>
       </c>
     </row>
@@ -2615,7 +2580,7 @@
       <c r="C4" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="15" t="s">
         <v>49</v>
       </c>
     </row>
@@ -2655,15 +2620,15 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
     </row>
     <row r="2" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
@@ -2759,13 +2724,13 @@
       <c r="D3" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="E3" s="15" t="n">
+      <c r="E3" s="16" t="n">
         <v>24</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="G3" s="9" t="s">
         <v>58</v>
       </c>
       <c r="H3" s="12"/>
@@ -2840,13 +2805,13 @@
       <c r="D4" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="E4" s="15" t="n">
+      <c r="E4" s="16" t="n">
         <v>12</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G4" s="16" t="s">
+      <c r="G4" s="9" t="s">
         <v>61</v>
       </c>
       <c r="H4" s="12"/>

</xml_diff>

<commit_message>
Solve simulation stream issue
</commit_message>
<xml_diff>
--- a/src/flychams_common/config/Configuration-Heterogeneous-Benchmark.xlsx
+++ b/src/flychams_common/config/Configuration-Heterogeneous-Benchmark.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -830,11 +830,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="h:mm:ss"/>
     <numFmt numFmtId="166" formatCode="0"/>
-    <numFmt numFmtId="167" formatCode="General"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -1004,7 +1003,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1098,10 +1097,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1414,37 +1409,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546a"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="e7e6e6"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472c4"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ed7d31"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a5a5a5"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="ffc000"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5b9bd5"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70ad47"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563c1"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954f72"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office 2013 - 2022">
@@ -1584,7 +1579,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:XFD11"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="21" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="21" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26.44"/>
@@ -2117,7 +2112,7 @@
       <c r="BD8" s="12"/>
     </row>
     <row r="9" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8"/>
+      <c r="A9" s="13"/>
       <c r="B9" s="9" t="s">
         <v>34</v>
       </c>
@@ -2195,7 +2190,7 @@
       <c r="BD9" s="12"/>
     </row>
     <row r="10" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8"/>
+      <c r="A10" s="13"/>
       <c r="B10" s="9" t="s">
         <v>37</v>
       </c>
@@ -2375,7 +2370,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="2" width="29.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="40.25"/>
@@ -2447,21 +2442,21 @@
       <c r="B3" s="23" t="s">
         <v>261</v>
       </c>
-      <c r="C3" s="24" t="b">
+      <c r="C3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="D3" s="23" t="s">
         <v>262</v>
       </c>
-      <c r="E3" s="24" t="b">
+      <c r="E3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="F3" s="23" t="s">
         <v>263</v>
       </c>
-      <c r="G3" s="24" t="b">
+      <c r="G3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2515,7 +2510,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.78"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="33.54"/>
@@ -2606,7 +2601,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:BM1048576"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="42.01"/>
@@ -2978,7 +2973,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD13"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="12" width="38.28"/>
@@ -3334,7 +3329,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="12" width="38.28"/>
@@ -3629,7 +3624,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD19"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="27.35"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="45.28"/>
@@ -4381,7 +4376,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD17"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="27.35"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="57.21"/>
@@ -4643,7 +4638,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:R1048576"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="34.63"/>
@@ -4754,28 +4749,28 @@
       <c r="E3" s="23" t="n">
         <v>12</v>
       </c>
-      <c r="F3" s="24" t="b">
+      <c r="F3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="G3" s="23" t="s">
         <v>233</v>
       </c>
-      <c r="H3" s="24" t="b">
+      <c r="H3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I3" s="23" t="s">
         <v>234</v>
       </c>
-      <c r="J3" s="24" t="b">
+      <c r="J3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="K3" s="23" t="s">
         <v>235</v>
       </c>
-      <c r="L3" s="24" t="b">
+      <c r="L3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -4838,7 +4833,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="63.93"/>
@@ -4925,7 +4920,7 @@
       <c r="F3" s="23" t="s">
         <v>249</v>
       </c>
-      <c r="G3" s="24" t="b">
+      <c r="G3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -4961,7 +4956,7 @@
       <c r="F4" s="23" t="s">
         <v>249</v>
       </c>
-      <c r="G4" s="24" t="b">
+      <c r="G4" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -4997,7 +4992,7 @@
       <c r="F5" s="23" t="s">
         <v>249</v>
       </c>
-      <c r="G5" s="24" t="b">
+      <c r="G5" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Fix normalized upsilon calculation
</commit_message>
<xml_diff>
--- a/src/flychams_common/config/Configuration-Heterogeneous-Benchmark.xlsx
+++ b/src/flychams_common/config/Configuration-Heterogeneous-Benchmark.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -830,12 +830,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="h:mm:ss"/>
     <numFmt numFmtId="166" formatCode="0"/>
+    <numFmt numFmtId="167" formatCode="General"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -903,13 +904,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="16"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">
@@ -1056,10 +1050,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1097,6 +1087,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1409,37 +1403,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="44546a"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="e7e6e6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4472c4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="ed7d31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="a5a5a5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="ffc000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="5b9bd5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="70ad47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0563c1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="954f72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office 2013 - 2022">
@@ -1579,7 +1573,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:XFD11"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="21" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="21" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26.44"/>
@@ -2112,7 +2106,7 @@
       <c r="BD8" s="12"/>
     </row>
     <row r="9" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13"/>
+      <c r="A9" s="8"/>
       <c r="B9" s="9" t="s">
         <v>34</v>
       </c>
@@ -2190,7 +2184,7 @@
       <c r="BD9" s="12"/>
     </row>
     <row r="10" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="13"/>
+      <c r="A10" s="8"/>
       <c r="B10" s="9" t="s">
         <v>37</v>
       </c>
@@ -2268,7 +2262,7 @@
       <c r="BD10" s="12"/>
     </row>
     <row r="11" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13" t="s">
+      <c r="A11" s="8" t="s">
         <v>39</v>
       </c>
       <c r="B11" s="9" t="s">
@@ -2370,7 +2364,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="2" width="29.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="40.25"/>
@@ -2384,92 +2378,92 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="20" t="s">
         <v>215</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="22" t="s">
+      <c r="C2" s="21" t="s">
         <v>255</v>
       </c>
-      <c r="D2" s="22" t="s">
+      <c r="D2" s="21" t="s">
         <v>256</v>
       </c>
-      <c r="E2" s="22" t="s">
+      <c r="E2" s="21" t="s">
         <v>257</v>
       </c>
-      <c r="F2" s="22" t="s">
+      <c r="F2" s="21" t="s">
         <v>258</v>
       </c>
-      <c r="G2" s="22" t="s">
+      <c r="G2" s="21" t="s">
         <v>259</v>
       </c>
-      <c r="H2" s="22" t="s">
+      <c r="H2" s="21" t="s">
         <v>260</v>
       </c>
-      <c r="I2" s="22" t="s">
+      <c r="I2" s="21" t="s">
         <v>242</v>
       </c>
-      <c r="J2" s="22" t="s">
+      <c r="J2" s="21" t="s">
         <v>243</v>
       </c>
-      <c r="K2" s="22" t="s">
+      <c r="K2" s="21" t="s">
         <v>244</v>
       </c>
       <c r="L2" s="12"/>
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="22" t="s">
         <v>132</v>
       </c>
-      <c r="B3" s="23" t="s">
+      <c r="B3" s="22" t="s">
         <v>261</v>
       </c>
       <c r="C3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="D3" s="23" t="s">
+      <c r="D3" s="22" t="s">
         <v>262</v>
       </c>
       <c r="E3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="F3" s="23" t="s">
+      <c r="F3" s="22" t="s">
         <v>263</v>
       </c>
       <c r="G3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H3" s="23" t="s">
+      <c r="H3" s="22" t="s">
         <v>264</v>
       </c>
-      <c r="I3" s="23" t="n">
+      <c r="I3" s="22" t="n">
         <v>0.4</v>
       </c>
-      <c r="J3" s="23" t="n">
+      <c r="J3" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="K3" s="23" t="n">
+      <c r="K3" s="22" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2510,7 +2504,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.78"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="33.54"/>
@@ -2523,12 +2517,12 @@
   </cols>
   <sheetData>
     <row r="1" s="7" customFormat="true" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
       <c r="E1" s="12"/>
       <c r="XFB1" s="3"/>
       <c r="XFC1" s="3"/>
@@ -2558,7 +2552,7 @@
       <c r="C3" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="14" t="s">
         <v>46</v>
       </c>
     </row>
@@ -2572,7 +2566,7 @@
       <c r="C4" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="14" t="s">
         <v>49</v>
       </c>
     </row>
@@ -2601,7 +2595,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:BM1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="42.01"/>
@@ -2612,15 +2606,15 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
     </row>
     <row r="2" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
@@ -2716,7 +2710,7 @@
       <c r="D3" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="E3" s="16" t="n">
+      <c r="E3" s="15" t="n">
         <v>24</v>
       </c>
       <c r="F3" s="9" t="s">
@@ -2797,7 +2791,7 @@
       <c r="D4" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="E4" s="16" t="n">
+      <c r="E4" s="15" t="n">
         <v>12</v>
       </c>
       <c r="F4" s="9" t="s">
@@ -2877,7 +2871,7 @@
       <c r="D5" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="E5" s="17" t="n">
+      <c r="E5" s="16" t="n">
         <v>18</v>
       </c>
       <c r="F5" s="9" t="s">
@@ -2973,7 +2967,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD13"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="12" width="38.28"/>
@@ -2992,48 +2986,48 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="19" t="s">
+      <c r="D2" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="E2" s="19" t="s">
+      <c r="E2" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="F2" s="19" t="s">
+      <c r="F2" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="G2" s="19" t="s">
+      <c r="G2" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="H2" s="19" t="s">
+      <c r="H2" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="I2" s="19" t="s">
+      <c r="I2" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="J2" s="19" t="s">
+      <c r="J2" s="18" t="s">
         <v>72</v>
       </c>
       <c r="L2" s="12"/>
@@ -3048,258 +3042,258 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="D3" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="E3" s="20" t="s">
+      <c r="E3" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="F3" s="20" t="s">
+      <c r="F3" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="G3" s="20" t="s">
+      <c r="G3" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="H3" s="20" t="n">
+      <c r="H3" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I3" s="20" t="n">
+      <c r="I3" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J3" s="20" t="n">
+      <c r="J3" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="19" t="s">
         <v>79</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="19" t="s">
         <v>80</v>
       </c>
-      <c r="C4" s="20" t="s">
+      <c r="C4" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="20" t="s">
+      <c r="D4" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="E4" s="20" t="s">
+      <c r="E4" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="F4" s="20" t="s">
+      <c r="F4" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="G4" s="20" t="s">
+      <c r="G4" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="H4" s="20" t="n">
+      <c r="H4" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I4" s="20" t="n">
+      <c r="I4" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J4" s="20" t="n">
+      <c r="J4" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="19" t="s">
         <v>84</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="E5" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="F5" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="G5" s="20" t="s">
+      <c r="G5" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="H5" s="20" t="n">
+      <c r="H5" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I5" s="20" t="n">
+      <c r="I5" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J5" s="20" t="n">
+      <c r="J5" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="C6" s="20" t="s">
+      <c r="C6" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="E6" s="20" t="s">
+      <c r="E6" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="F6" s="20" t="s">
+      <c r="F6" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="G6" s="20" t="s">
+      <c r="G6" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="H6" s="20" t="n">
+      <c r="H6" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I6" s="20" t="n">
+      <c r="I6" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J6" s="20" t="n">
+      <c r="J6" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="20" t="s">
+      <c r="A7" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="B7" s="20" t="s">
+      <c r="B7" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="C7" s="20" t="s">
+      <c r="C7" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="D7" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="E7" s="20" t="s">
+      <c r="E7" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="F7" s="20" t="s">
+      <c r="F7" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="G7" s="20" t="s">
+      <c r="G7" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="H7" s="20" t="n">
+      <c r="H7" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I7" s="20" t="n">
+      <c r="I7" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J7" s="20" t="n">
+      <c r="J7" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="20" t="s">
+      <c r="A8" s="19" t="s">
         <v>93</v>
       </c>
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="C8" s="20" t="s">
+      <c r="C8" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="D8" s="19" t="s">
         <v>95</v>
       </c>
-      <c r="E8" s="20" t="s">
+      <c r="E8" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="F8" s="20" t="s">
+      <c r="F8" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="G8" s="20" t="s">
+      <c r="G8" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="H8" s="20" t="n">
+      <c r="H8" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I8" s="20" t="n">
+      <c r="I8" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J8" s="20" t="n">
+      <c r="J8" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="20" t="s">
+      <c r="A9" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="B9" s="20" t="s">
+      <c r="B9" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="C9" s="20" t="s">
+      <c r="C9" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="20" t="s">
+      <c r="D9" s="19" t="s">
         <v>98</v>
       </c>
-      <c r="E9" s="20" t="s">
+      <c r="E9" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="F9" s="20" t="s">
+      <c r="F9" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="G9" s="20" t="s">
+      <c r="G9" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="H9" s="20" t="n">
+      <c r="H9" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I9" s="20" t="n">
+      <c r="I9" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J9" s="20" t="n">
+      <c r="J9" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="B10" s="20" t="s">
+      <c r="B10" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="C10" s="20" t="s">
+      <c r="C10" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="20" t="s">
+      <c r="D10" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="E10" s="20" t="s">
+      <c r="E10" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="F10" s="20" t="s">
+      <c r="F10" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="G10" s="20" t="s">
+      <c r="G10" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="20" t="n">
+      <c r="H10" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I10" s="20" t="n">
+      <c r="I10" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J10" s="20" t="n">
+      <c r="J10" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
@@ -3329,7 +3323,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="12" width="38.28"/>
@@ -3345,32 +3339,32 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="D2" s="19" t="s">
+      <c r="D2" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="E2" s="19" t="s">
+      <c r="E2" s="18" t="s">
         <v>104</v>
       </c>
-      <c r="F2" s="19" t="s">
+      <c r="F2" s="18" t="s">
         <v>105</v>
       </c>
       <c r="H2" s="12"/>
@@ -3386,22 +3380,22 @@
       <c r="XFD2" s="12"/>
     </row>
     <row r="3" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="D3" s="20" t="n">
+      <c r="D3" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E3" s="20" t="n">
+      <c r="E3" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F3" s="20" t="n">
+      <c r="F3" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G3" s="2"/>
@@ -3411,22 +3405,22 @@
       <c r="XEY3" s="3"/>
     </row>
     <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="C4" s="20" t="s">
+      <c r="C4" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="D4" s="20" t="n">
+      <c r="D4" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E4" s="20" t="n">
+      <c r="E4" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F4" s="20" t="n">
+      <c r="F4" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G4" s="2"/>
@@ -3436,22 +3430,22 @@
       <c r="XEY4" s="3"/>
     </row>
     <row r="5" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="19" t="s">
         <v>110</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="D5" s="20" t="n">
+      <c r="D5" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E5" s="20" t="n">
+      <c r="E5" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F5" s="20" t="n">
+      <c r="F5" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G5" s="2"/>
@@ -3461,22 +3455,22 @@
       <c r="XEY5" s="3"/>
     </row>
     <row r="6" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C6" s="20" t="s">
+      <c r="C6" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="D6" s="20" t="n">
+      <c r="D6" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E6" s="20" t="n">
+      <c r="E6" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F6" s="20" t="n">
+      <c r="F6" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G6" s="2"/>
@@ -3486,22 +3480,22 @@
       <c r="XEY6" s="3"/>
     </row>
     <row r="7" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="20" t="s">
+      <c r="A7" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="B7" s="20" t="s">
+      <c r="B7" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="C7" s="20" t="s">
+      <c r="C7" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="D7" s="20" t="n">
+      <c r="D7" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E7" s="20" t="n">
+      <c r="E7" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F7" s="20" t="n">
+      <c r="F7" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G7" s="2"/>
@@ -3511,22 +3505,22 @@
       <c r="XEY7" s="3"/>
     </row>
     <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="20" t="s">
+      <c r="A8" s="19" t="s">
         <v>95</v>
       </c>
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="19" t="s">
         <v>116</v>
       </c>
-      <c r="C8" s="20" t="s">
+      <c r="C8" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="D8" s="20" t="n">
+      <c r="D8" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E8" s="20" t="n">
+      <c r="E8" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F8" s="20" t="n">
+      <c r="F8" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G8" s="2"/>
@@ -3536,22 +3530,22 @@
       <c r="XEY8" s="3"/>
     </row>
     <row r="9" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="20" t="s">
+      <c r="A9" s="19" t="s">
         <v>98</v>
       </c>
-      <c r="B9" s="20" t="s">
+      <c r="B9" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="C9" s="20" t="s">
+      <c r="C9" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="D9" s="20" t="n">
+      <c r="D9" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E9" s="20" t="n">
+      <c r="E9" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F9" s="20" t="n">
+      <c r="F9" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G9" s="2"/>
@@ -3561,22 +3555,22 @@
       <c r="XEY9" s="3"/>
     </row>
     <row r="10" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="B10" s="20" t="s">
+      <c r="B10" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="C10" s="20" t="s">
+      <c r="C10" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="D10" s="20" t="n">
+      <c r="D10" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E10" s="20" t="n">
+      <c r="E10" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F10" s="20" t="n">
+      <c r="F10" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G10" s="2"/>
@@ -3624,7 +3618,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD19"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="27.35"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="45.28"/>
@@ -3642,56 +3636,56 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="D2" s="19" t="s">
+      <c r="D2" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="E2" s="19" t="s">
+      <c r="E2" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="F2" s="19" t="s">
+      <c r="F2" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="G2" s="19" t="s">
+      <c r="G2" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="H2" s="19" t="s">
+      <c r="H2" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="I2" s="19" t="s">
+      <c r="I2" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="J2" s="19" t="s">
+      <c r="J2" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="K2" s="19" t="s">
+      <c r="K2" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="L2" s="19" t="s">
+      <c r="L2" s="18" t="s">
         <v>128</v>
       </c>
       <c r="M2" s="12"/>
@@ -3704,652 +3698,652 @@
       <c r="XFC2" s="12"/>
     </row>
     <row r="3" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="19" t="s">
         <v>129</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="19" t="s">
         <v>130</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="D3" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="E3" s="20" t="s">
+      <c r="E3" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F3" s="20" t="s">
+      <c r="F3" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="G3" s="20" t="s">
+      <c r="G3" s="19" t="s">
         <v>134</v>
       </c>
-      <c r="H3" s="20" t="s">
+      <c r="H3" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="I3" s="20" t="n">
+      <c r="I3" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J3" s="20" t="n">
+      <c r="J3" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="K3" s="20" t="n">
+      <c r="K3" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L3" s="20" t="s">
+      <c r="L3" s="19" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="19" t="s">
         <v>137</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="19" t="s">
         <v>138</v>
       </c>
-      <c r="C4" s="20" t="s">
+      <c r="C4" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="D4" s="20" t="s">
+      <c r="D4" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="E4" s="20" t="s">
+      <c r="E4" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F4" s="20" t="s">
+      <c r="F4" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="G4" s="20" t="s">
+      <c r="G4" s="19" t="s">
         <v>141</v>
       </c>
-      <c r="H4" s="20" t="s">
+      <c r="H4" s="19" t="s">
         <v>142</v>
       </c>
-      <c r="I4" s="20" t="n">
+      <c r="I4" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J4" s="20" t="n">
+      <c r="J4" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K4" s="20" t="n">
+      <c r="K4" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L4" s="20" t="s">
+      <c r="L4" s="19" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="19" t="s">
         <v>144</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="19" t="s">
         <v>145</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="E5" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="F5" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="G5" s="20" t="s">
+      <c r="G5" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="H5" s="20" t="s">
+      <c r="H5" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="I5" s="20" t="n">
+      <c r="I5" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J5" s="20" t="n">
+      <c r="J5" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K5" s="20" t="n">
+      <c r="K5" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L5" s="20" t="s">
+      <c r="L5" s="19" t="s">
         <v>148</v>
       </c>
       <c r="XFD5" s="12"/>
     </row>
     <row r="6" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="19" t="s">
         <v>149</v>
       </c>
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="19" t="s">
         <v>150</v>
       </c>
-      <c r="C6" s="20" t="s">
+      <c r="C6" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="E6" s="20" t="s">
+      <c r="E6" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F6" s="20" t="s">
+      <c r="F6" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="G6" s="20" t="s">
+      <c r="G6" s="19" t="s">
         <v>134</v>
       </c>
-      <c r="H6" s="20" t="s">
+      <c r="H6" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="I6" s="20" t="n">
+      <c r="I6" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J6" s="20" t="n">
+      <c r="J6" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="K6" s="20" t="n">
+      <c r="K6" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L6" s="20" t="s">
+      <c r="L6" s="19" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="7" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="20" t="s">
+      <c r="A7" s="19" t="s">
         <v>152</v>
       </c>
-      <c r="B7" s="20" t="s">
+      <c r="B7" s="19" t="s">
         <v>153</v>
       </c>
-      <c r="C7" s="20" t="s">
+      <c r="C7" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="D7" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="E7" s="20" t="s">
+      <c r="E7" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F7" s="20" t="s">
+      <c r="F7" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="G7" s="20" t="s">
+      <c r="G7" s="19" t="s">
         <v>141</v>
       </c>
-      <c r="H7" s="20" t="s">
+      <c r="H7" s="19" t="s">
         <v>142</v>
       </c>
-      <c r="I7" s="20" t="n">
+      <c r="I7" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J7" s="20" t="n">
+      <c r="J7" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K7" s="20" t="n">
+      <c r="K7" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L7" s="20" t="s">
+      <c r="L7" s="19" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="20" t="s">
+      <c r="A8" s="19" t="s">
         <v>155</v>
       </c>
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="19" t="s">
         <v>156</v>
       </c>
-      <c r="C8" s="20" t="s">
+      <c r="C8" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="D8" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="E8" s="20" t="s">
+      <c r="E8" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F8" s="20" t="s">
+      <c r="F8" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="G8" s="20" t="s">
+      <c r="G8" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="H8" s="20" t="s">
+      <c r="H8" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="I8" s="20" t="n">
+      <c r="I8" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J8" s="20" t="n">
+      <c r="J8" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K8" s="20" t="n">
+      <c r="K8" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L8" s="20" t="s">
+      <c r="L8" s="19" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="9" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="20" t="s">
+      <c r="A9" s="19" t="s">
         <v>158</v>
       </c>
-      <c r="B9" s="20" t="s">
+      <c r="B9" s="19" t="s">
         <v>159</v>
       </c>
-      <c r="C9" s="20" t="s">
+      <c r="C9" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="D9" s="20" t="s">
+      <c r="D9" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="E9" s="20" t="s">
+      <c r="E9" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F9" s="20" t="s">
+      <c r="F9" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="G9" s="20" t="s">
+      <c r="G9" s="19" t="s">
         <v>134</v>
       </c>
-      <c r="H9" s="20" t="s">
+      <c r="H9" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="I9" s="20" t="n">
+      <c r="I9" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J9" s="20" t="n">
+      <c r="J9" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="K9" s="20" t="n">
+      <c r="K9" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L9" s="20" t="s">
+      <c r="L9" s="19" t="s">
         <v>160</v>
       </c>
       <c r="XFD9" s="2"/>
     </row>
     <row r="10" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="19" t="s">
         <v>161</v>
       </c>
-      <c r="B10" s="20" t="s">
+      <c r="B10" s="19" t="s">
         <v>162</v>
       </c>
-      <c r="C10" s="20" t="s">
+      <c r="C10" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="D10" s="20" t="s">
+      <c r="D10" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="E10" s="20" t="s">
+      <c r="E10" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F10" s="20" t="s">
+      <c r="F10" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="G10" s="20" t="s">
+      <c r="G10" s="19" t="s">
         <v>141</v>
       </c>
-      <c r="H10" s="20" t="s">
+      <c r="H10" s="19" t="s">
         <v>142</v>
       </c>
-      <c r="I10" s="20" t="n">
+      <c r="I10" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J10" s="20" t="n">
+      <c r="J10" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K10" s="20" t="n">
+      <c r="K10" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L10" s="20" t="s">
+      <c r="L10" s="19" t="s">
         <v>163</v>
       </c>
       <c r="XFD10" s="2"/>
     </row>
     <row r="11" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="20" t="s">
+      <c r="A11" s="19" t="s">
         <v>164</v>
       </c>
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="19" t="s">
         <v>165</v>
       </c>
-      <c r="C11" s="20" t="s">
+      <c r="C11" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="D11" s="20" t="s">
+      <c r="D11" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="E11" s="20" t="s">
+      <c r="E11" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F11" s="20" t="s">
+      <c r="F11" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="G11" s="20" t="s">
+      <c r="G11" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="H11" s="20" t="s">
+      <c r="H11" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="I11" s="20" t="n">
+      <c r="I11" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J11" s="20" t="n">
+      <c r="J11" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K11" s="20" t="n">
+      <c r="K11" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L11" s="20" t="s">
+      <c r="L11" s="19" t="s">
         <v>166</v>
       </c>
       <c r="XFD11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="20" t="s">
+      <c r="A12" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="B12" s="20" t="s">
+      <c r="B12" s="19" t="s">
         <v>168</v>
       </c>
-      <c r="C12" s="20" t="s">
+      <c r="C12" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="D12" s="20" t="s">
+      <c r="D12" s="19" t="s">
         <v>169</v>
       </c>
-      <c r="E12" s="20" t="s">
+      <c r="E12" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F12" s="20" t="s">
+      <c r="F12" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="G12" s="20" t="s">
+      <c r="G12" s="19" t="s">
         <v>141</v>
       </c>
-      <c r="H12" s="20" t="s">
+      <c r="H12" s="19" t="s">
         <v>142</v>
       </c>
-      <c r="I12" s="20" t="n">
+      <c r="I12" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J12" s="20" t="n">
+      <c r="J12" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="K12" s="20" t="n">
+      <c r="K12" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L12" s="20" t="s">
+      <c r="L12" s="19" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="20" t="s">
+      <c r="A13" s="19" t="s">
         <v>171</v>
       </c>
-      <c r="B13" s="20" t="s">
+      <c r="B13" s="19" t="s">
         <v>172</v>
       </c>
-      <c r="C13" s="20" t="s">
+      <c r="C13" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="D13" s="20" t="s">
+      <c r="D13" s="19" t="s">
         <v>169</v>
       </c>
-      <c r="E13" s="20" t="s">
+      <c r="E13" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F13" s="20" t="s">
+      <c r="F13" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="G13" s="20" t="s">
+      <c r="G13" s="19" t="s">
         <v>141</v>
       </c>
-      <c r="H13" s="20" t="s">
+      <c r="H13" s="19" t="s">
         <v>142</v>
       </c>
-      <c r="I13" s="20" t="n">
+      <c r="I13" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J13" s="20" t="n">
+      <c r="J13" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="K13" s="20" t="n">
+      <c r="K13" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L13" s="20" t="s">
+      <c r="L13" s="19" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20" t="s">
+      <c r="A14" s="19" t="s">
         <v>174</v>
       </c>
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="19" t="s">
         <v>175</v>
       </c>
-      <c r="C14" s="20" t="s">
+      <c r="C14" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="D14" s="20" t="s">
+      <c r="D14" s="19" t="s">
         <v>169</v>
       </c>
-      <c r="E14" s="20" t="s">
+      <c r="E14" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F14" s="20" t="s">
+      <c r="F14" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="G14" s="20" t="s">
+      <c r="G14" s="19" t="s">
         <v>141</v>
       </c>
-      <c r="H14" s="20" t="s">
+      <c r="H14" s="19" t="s">
         <v>142</v>
       </c>
-      <c r="I14" s="20" t="n">
+      <c r="I14" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J14" s="20" t="n">
+      <c r="J14" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="K14" s="20" t="n">
+      <c r="K14" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L14" s="20" t="s">
+      <c r="L14" s="19" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="20" t="s">
+      <c r="A15" s="19" t="s">
         <v>177</v>
       </c>
-      <c r="B15" s="20" t="s">
+      <c r="B15" s="19" t="s">
         <v>178</v>
       </c>
-      <c r="C15" s="20" t="s">
+      <c r="C15" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="D15" s="20" t="s">
+      <c r="D15" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="E15" s="20" t="s">
+      <c r="E15" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F15" s="20" t="s">
+      <c r="F15" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="G15" s="20" t="s">
+      <c r="G15" s="19" t="s">
         <v>134</v>
       </c>
-      <c r="H15" s="20" t="s">
+      <c r="H15" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="I15" s="20" t="n">
+      <c r="I15" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J15" s="20" t="n">
+      <c r="J15" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="K15" s="20" t="n">
+      <c r="K15" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L15" s="20" t="s">
+      <c r="L15" s="19" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="20" t="s">
+      <c r="A16" s="19" t="s">
         <v>180</v>
       </c>
-      <c r="B16" s="20" t="s">
+      <c r="B16" s="19" t="s">
         <v>181</v>
       </c>
-      <c r="C16" s="20" t="s">
+      <c r="C16" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="D16" s="20" t="s">
+      <c r="D16" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="E16" s="20" t="s">
+      <c r="E16" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F16" s="20" t="s">
+      <c r="F16" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="G16" s="20" t="s">
+      <c r="G16" s="19" t="s">
         <v>141</v>
       </c>
-      <c r="H16" s="20" t="s">
+      <c r="H16" s="19" t="s">
         <v>142</v>
       </c>
-      <c r="I16" s="20" t="n">
+      <c r="I16" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J16" s="20" t="n">
+      <c r="J16" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K16" s="20" t="n">
+      <c r="K16" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L16" s="20" t="s">
+      <c r="L16" s="19" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="20" t="s">
+      <c r="A17" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="B17" s="20" t="s">
+      <c r="B17" s="19" t="s">
         <v>184</v>
       </c>
-      <c r="C17" s="20" t="s">
+      <c r="C17" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="D17" s="20" t="s">
+      <c r="D17" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="E17" s="20" t="s">
+      <c r="E17" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F17" s="20" t="s">
+      <c r="F17" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="G17" s="20" t="s">
+      <c r="G17" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="H17" s="20" t="s">
+      <c r="H17" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="I17" s="20" t="n">
+      <c r="I17" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J17" s="20" t="n">
+      <c r="J17" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K17" s="20" t="n">
+      <c r="K17" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L17" s="20" t="s">
+      <c r="L17" s="19" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="20" t="s">
+      <c r="A18" s="19" t="s">
         <v>186</v>
       </c>
-      <c r="B18" s="20" t="s">
+      <c r="B18" s="19" t="s">
         <v>187</v>
       </c>
-      <c r="C18" s="20" t="s">
+      <c r="C18" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="D18" s="20" t="s">
+      <c r="D18" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="E18" s="20" t="s">
+      <c r="E18" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F18" s="20" t="s">
+      <c r="F18" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="G18" s="20" t="s">
+      <c r="G18" s="19" t="s">
         <v>188</v>
       </c>
-      <c r="H18" s="20" t="s">
+      <c r="H18" s="19" t="s">
         <v>189</v>
       </c>
-      <c r="I18" s="20" t="n">
+      <c r="I18" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J18" s="20" t="n">
+      <c r="J18" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K18" s="20" t="n">
+      <c r="K18" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L18" s="20" t="s">
+      <c r="L18" s="19" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="20" t="s">
+      <c r="A19" s="19" t="s">
         <v>191</v>
       </c>
-      <c r="B19" s="20" t="s">
+      <c r="B19" s="19" t="s">
         <v>192</v>
       </c>
-      <c r="C19" s="20" t="s">
+      <c r="C19" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="D19" s="20" t="s">
+      <c r="D19" s="19" t="s">
         <v>169</v>
       </c>
-      <c r="E19" s="20" t="s">
+      <c r="E19" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F19" s="20" t="s">
+      <c r="F19" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="G19" s="20" t="s">
+      <c r="G19" s="19" t="s">
         <v>141</v>
       </c>
-      <c r="H19" s="20" t="s">
+      <c r="H19" s="19" t="s">
         <v>142</v>
       </c>
-      <c r="I19" s="20" t="n">
+      <c r="I19" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J19" s="20" t="n">
+      <c r="J19" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="K19" s="20" t="n">
+      <c r="K19" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L19" s="20" t="s">
+      <c r="L19" s="19" t="s">
         <v>193</v>
       </c>
     </row>
@@ -4376,7 +4370,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD17"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="27.35"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="57.21"/>
@@ -4389,32 +4383,32 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="D2" s="19" t="s">
+      <c r="D2" s="18" t="s">
         <v>194</v>
       </c>
-      <c r="E2" s="19" t="s">
+      <c r="E2" s="18" t="s">
         <v>195</v>
       </c>
-      <c r="F2" s="19" t="s">
+      <c r="F2" s="18" t="s">
         <v>196</v>
       </c>
       <c r="XET2" s="3"/>
@@ -4430,182 +4424,182 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="19" t="s">
         <v>197</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="D3" s="20" t="n">
+      <c r="D3" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="E3" s="20" t="n">
+      <c r="E3" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="F3" s="20" t="n">
+      <c r="F3" s="19" t="n">
         <v>0.625</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="19" t="s">
         <v>200</v>
       </c>
-      <c r="C4" s="20" t="s">
+      <c r="C4" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="D4" s="20" t="n">
+      <c r="D4" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="E4" s="20" t="n">
+      <c r="E4" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="F4" s="20" t="n">
+      <c r="F4" s="19" t="n">
         <v>0.625</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="19" t="s">
         <v>201</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="19" t="s">
         <v>202</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="D5" s="20" t="n">
+      <c r="D5" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="E5" s="20" t="n">
+      <c r="E5" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="20" t="n">
+      <c r="F5" s="19" t="n">
         <v>0.625</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="19" t="s">
         <v>203</v>
       </c>
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="19" t="s">
         <v>204</v>
       </c>
-      <c r="C6" s="20" t="s">
+      <c r="C6" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="D6" s="20" t="n">
+      <c r="D6" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="E6" s="20" t="n">
+      <c r="E6" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="20" t="n">
+      <c r="F6" s="19" t="n">
         <v>0.625</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="20" t="s">
+      <c r="A7" s="19" t="s">
         <v>205</v>
       </c>
-      <c r="B7" s="20" t="s">
+      <c r="B7" s="19" t="s">
         <v>206</v>
       </c>
-      <c r="C7" s="20" t="s">
+      <c r="C7" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="D7" s="20" t="n">
+      <c r="D7" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="E7" s="20" t="n">
+      <c r="E7" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="20" t="n">
+      <c r="F7" s="19" t="n">
         <v>0.625</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="20" t="s">
+      <c r="A8" s="19" t="s">
         <v>207</v>
       </c>
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="19" t="s">
         <v>208</v>
       </c>
-      <c r="C8" s="20" t="s">
+      <c r="C8" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="D8" s="20" t="n">
+      <c r="D8" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="E8" s="20" t="n">
+      <c r="E8" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="20" t="n">
+      <c r="F8" s="19" t="n">
         <v>0.625</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="20" t="s">
+      <c r="A9" s="19" t="s">
         <v>209</v>
       </c>
-      <c r="B9" s="20" t="s">
+      <c r="B9" s="19" t="s">
         <v>210</v>
       </c>
-      <c r="C9" s="20" t="s">
+      <c r="C9" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="D9" s="20" t="n">
+      <c r="D9" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="E9" s="20" t="n">
+      <c r="E9" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="20" t="n">
+      <c r="F9" s="19" t="n">
         <v>0.625</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="19" t="s">
         <v>211</v>
       </c>
-      <c r="B10" s="20" t="s">
+      <c r="B10" s="19" t="s">
         <v>212</v>
       </c>
-      <c r="C10" s="20" t="s">
+      <c r="C10" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="D10" s="20" t="n">
+      <c r="D10" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="E10" s="20" t="n">
+      <c r="E10" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="F10" s="20" t="n">
+      <c r="F10" s="19" t="n">
         <v>0.625</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="20" t="s">
+      <c r="A11" s="19" t="s">
         <v>213</v>
       </c>
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="19" t="s">
         <v>214</v>
       </c>
-      <c r="C11" s="20" t="s">
+      <c r="C11" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="D11" s="20" t="n">
+      <c r="D11" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="E11" s="20" t="n">
+      <c r="E11" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="20" t="n">
+      <c r="F11" s="19" t="n">
         <v>0.625</v>
       </c>
     </row>
@@ -4638,7 +4632,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:R1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="34.63"/>
@@ -4656,140 +4650,140 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="20" t="s">
         <v>215</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-      <c r="L1" s="21"/>
-      <c r="M1" s="21"/>
-      <c r="N1" s="21"/>
-      <c r="O1" s="21"/>
-      <c r="P1" s="21"/>
-      <c r="Q1" s="21"/>
-      <c r="R1" s="21"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="20"/>
+      <c r="N1" s="20"/>
+      <c r="O1" s="20"/>
+      <c r="P1" s="20"/>
+      <c r="Q1" s="20"/>
+      <c r="R1" s="20"/>
     </row>
     <row r="2" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="22" t="s">
+      <c r="C2" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="D2" s="22" t="s">
+      <c r="D2" s="21" t="s">
         <v>216</v>
       </c>
-      <c r="E2" s="22" t="s">
+      <c r="E2" s="21" t="s">
         <v>217</v>
       </c>
-      <c r="F2" s="22" t="s">
+      <c r="F2" s="21" t="s">
         <v>218</v>
       </c>
-      <c r="G2" s="22" t="s">
+      <c r="G2" s="21" t="s">
         <v>219</v>
       </c>
-      <c r="H2" s="22" t="s">
+      <c r="H2" s="21" t="s">
         <v>220</v>
       </c>
-      <c r="I2" s="22" t="s">
+      <c r="I2" s="21" t="s">
         <v>221</v>
       </c>
-      <c r="J2" s="22" t="s">
+      <c r="J2" s="21" t="s">
         <v>222</v>
       </c>
-      <c r="K2" s="22" t="s">
+      <c r="K2" s="21" t="s">
         <v>223</v>
       </c>
-      <c r="L2" s="22" t="s">
+      <c r="L2" s="21" t="s">
         <v>224</v>
       </c>
-      <c r="M2" s="22" t="s">
+      <c r="M2" s="21" t="s">
         <v>225</v>
       </c>
-      <c r="N2" s="22" t="s">
+      <c r="N2" s="21" t="s">
         <v>226</v>
       </c>
-      <c r="O2" s="22" t="s">
+      <c r="O2" s="21" t="s">
         <v>227</v>
       </c>
-      <c r="P2" s="22" t="s">
+      <c r="P2" s="21" t="s">
         <v>228</v>
       </c>
-      <c r="Q2" s="22" t="s">
+      <c r="Q2" s="21" t="s">
         <v>229</v>
       </c>
-      <c r="R2" s="22" t="s">
+      <c r="R2" s="21" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="B3" s="23" t="s">
+      <c r="B3" s="22" t="s">
         <v>231</v>
       </c>
-      <c r="C3" s="23" t="s">
+      <c r="C3" s="22" t="s">
         <v>232</v>
       </c>
-      <c r="D3" s="23" t="n">
+      <c r="D3" s="22" t="n">
         <v>8</v>
       </c>
-      <c r="E3" s="23" t="n">
+      <c r="E3" s="22" t="n">
         <v>12</v>
       </c>
       <c r="F3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="G3" s="23" t="s">
+      <c r="G3" s="22" t="s">
         <v>233</v>
       </c>
       <c r="H3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="I3" s="23" t="s">
+      <c r="I3" s="22" t="s">
         <v>234</v>
       </c>
       <c r="J3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="K3" s="23" t="s">
+      <c r="K3" s="22" t="s">
         <v>235</v>
       </c>
       <c r="L3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="M3" s="23" t="s">
+      <c r="M3" s="22" t="s">
         <v>236</v>
       </c>
-      <c r="N3" s="23" t="n">
+      <c r="N3" s="22" t="n">
         <v>6.5</v>
       </c>
-      <c r="O3" s="23" t="n">
+      <c r="O3" s="22" t="n">
         <v>2.5</v>
       </c>
-      <c r="P3" s="23" t="n">
+      <c r="P3" s="22" t="n">
         <v>400</v>
       </c>
-      <c r="Q3" s="23" t="n">
+      <c r="Q3" s="22" t="n">
         <v>350</v>
       </c>
-      <c r="R3" s="23" t="n">
+      <c r="R3" s="22" t="n">
         <v>25</v>
       </c>
     </row>
@@ -4833,7 +4827,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="63.93"/>
@@ -4849,52 +4843,52 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="20" t="s">
         <v>215</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="22" t="s">
+      <c r="C2" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="D2" s="22" t="s">
+      <c r="D2" s="21" t="s">
         <v>237</v>
       </c>
-      <c r="E2" s="22" t="s">
+      <c r="E2" s="21" t="s">
         <v>238</v>
       </c>
-      <c r="F2" s="22" t="s">
+      <c r="F2" s="21" t="s">
         <v>239</v>
       </c>
-      <c r="G2" s="22" t="s">
+      <c r="G2" s="21" t="s">
         <v>240</v>
       </c>
-      <c r="H2" s="22" t="s">
+      <c r="H2" s="21" t="s">
         <v>241</v>
       </c>
-      <c r="I2" s="22" t="s">
+      <c r="I2" s="21" t="s">
         <v>242</v>
       </c>
-      <c r="J2" s="22" t="s">
+      <c r="J2" s="21" t="s">
         <v>243</v>
       </c>
-      <c r="K2" s="22" t="s">
+      <c r="K2" s="21" t="s">
         <v>244</v>
       </c>
       <c r="XFB2" s="3"/>
@@ -4902,110 +4896,110 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="22" t="s">
         <v>131</v>
       </c>
-      <c r="B3" s="23" t="s">
+      <c r="B3" s="22" t="s">
         <v>245</v>
       </c>
-      <c r="C3" s="23" t="s">
+      <c r="C3" s="22" t="s">
         <v>246</v>
       </c>
-      <c r="D3" s="23" t="s">
+      <c r="D3" s="22" t="s">
         <v>247</v>
       </c>
-      <c r="E3" s="23" t="s">
+      <c r="E3" s="22" t="s">
         <v>248</v>
       </c>
-      <c r="F3" s="23" t="s">
+      <c r="F3" s="22" t="s">
         <v>249</v>
       </c>
       <c r="G3" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H3" s="23" t="s">
+      <c r="H3" s="22" t="s">
         <v>250</v>
       </c>
-      <c r="I3" s="23" t="n">
+      <c r="I3" s="22" t="n">
         <v>0.5</v>
       </c>
-      <c r="J3" s="23" t="n">
+      <c r="J3" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="K3" s="23" t="n">
+      <c r="K3" s="22" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="22" t="s">
         <v>251</v>
       </c>
-      <c r="C4" s="23" t="s">
+      <c r="C4" s="22" t="s">
         <v>246</v>
       </c>
-      <c r="D4" s="23" t="s">
+      <c r="D4" s="22" t="s">
         <v>252</v>
       </c>
-      <c r="E4" s="23" t="s">
+      <c r="E4" s="22" t="s">
         <v>248</v>
       </c>
-      <c r="F4" s="23" t="s">
+      <c r="F4" s="22" t="s">
         <v>249</v>
       </c>
       <c r="G4" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H4" s="23" t="s">
+      <c r="H4" s="22" t="s">
         <v>250</v>
       </c>
-      <c r="I4" s="23" t="n">
+      <c r="I4" s="22" t="n">
         <v>0.5</v>
       </c>
-      <c r="J4" s="23" t="n">
+      <c r="J4" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="K4" s="23" t="n">
+      <c r="K4" s="22" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="23" t="s">
+      <c r="A5" s="22" t="s">
         <v>169</v>
       </c>
-      <c r="B5" s="23" t="s">
+      <c r="B5" s="22" t="s">
         <v>253</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="C5" s="22" t="s">
         <v>246</v>
       </c>
-      <c r="D5" s="23" t="s">
+      <c r="D5" s="22" t="s">
         <v>254</v>
       </c>
-      <c r="E5" s="23" t="s">
+      <c r="E5" s="22" t="s">
         <v>248</v>
       </c>
-      <c r="F5" s="23" t="s">
+      <c r="F5" s="22" t="s">
         <v>249</v>
       </c>
       <c r="G5" s="23" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H5" s="23" t="s">
+      <c r="H5" s="22" t="s">
         <v>250</v>
       </c>
-      <c r="I5" s="23" t="n">
+      <c r="I5" s="22" t="n">
         <v>0.5</v>
       </c>
-      <c r="J5" s="23" t="n">
+      <c r="J5" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="K5" s="23" t="n">
+      <c r="K5" s="22" t="n">
         <v>5</v>
       </c>
     </row>

</xml_diff>